<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 2)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -660,8 +660,49 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1203285017</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>changmidang</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[Ultra Xecond Ski] パーフェクトヌード透明サンパッチ（ゴルフサンパッチ）10回分（計20枚）UVA&amp;amp;UVB強力遮断/日焼け止めパッチ/ゴルフパッチ/テニス/屋外スポーツ/紫外線</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Ultra Xecond Skin</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>3930</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203285017</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 3)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -701,8 +701,254 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1209641531</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[1+]NEWサイトカインブースタープロ 70ml＋70ml</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Refilled</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209641531</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1209148971</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>【韓国正規品/NEW】Gureum o de perfume EDP 50ml</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>11419</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209148971</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1206526891</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>[NEW]エアロクーリングシャンプー 400ml＋70ml / -5.2度急速冷却</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>3859</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206526891</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1207207330</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>COCOJI</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>【保湿・輝き・弾力】 PDR&amp;amp;N エッセンス 100 30ml ダブル企画</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>5794</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207207330</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1139814745</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>vip_s</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ティルティールオフザサンエアムース/ 40ml/ 1個</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>2247</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139814745</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1151569871</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>vip_s</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>デイリー アンチヘアロス タンパク質 トリートメント 500ml</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>3048</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151569871</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 6, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -947,8 +947,377 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1135668857</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>koco_store</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>[韓国人気保湿クリーム] グルカミュー(Glucamune)クリーム, 100ml (水分鎮静/スキンケア)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>5833</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135668857</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1187773893</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>trailblue2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>[25SS/New]コントロール-T ティーツリー ACクーリングクレンジングジェル 200ml (セラミドクレンジングフォーム 30ml 贈呈)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>リアルバリア</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>2834</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187773893</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1212343699</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pickary</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>【5枚入り】 垢すりグローブ ソフトボディ レッドグローブ クリーン角質ケア・ボディクレンジング 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212343699</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1192678454</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】 肌荒れ・乾燥くすみ対策に！エイシカ365 トラブルリリーフセラムpH4.5 40ml 肌荒れ くすみ 乾燥 美容液</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>2910</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192678454</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1192676012</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】アトバリア365 クリーム 80mL 保湿クリーム 水分クリーム 保湿カプセル セラミド クリーム 肌荒れ 水分</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>2470</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192676012</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1192160801</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>レチノール シカ リペア セラム 30mL</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192160801</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1135766293</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ChicAura</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ハイドロ セラミック トーンアップ エッセンス 日焼け止め 50ml</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>3727</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135766293</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1187174274</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ChicAura</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>[1+1] ディオルガ メディAHAクリーム 25ml 角質ケア×水分チャージ</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>3318</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187174274</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1185531865</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ChicAura</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>トラブルクリアpHバランストジェルクレンザー 200ml</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>2937</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185531865</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J12"/>
+  <autoFilter ref="A1:J21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 9, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1316,8 +1316,541 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1133764204</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>shintenchi</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>バイオコラーゲンリアルディープマスク, 4枚</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>2120</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133764204</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1207544119</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>shintenchi</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>エキスパートマデカクリームリニューPDRN, 50ml</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2330</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207544119</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1142629949</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>zozoro0213</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>セラ 水分バリア 日焼け止め SPF50+ PA++++ 50ml x 2個 (鎮静/弾力/保湿/栄養供給/活力/しわ防止)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>リアルバリア</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142629949</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1210932470</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ブルー EGF カーミングミスト 100ml 韓国フェイスミスト 化粧水ミスト うるおいケア 肌コンディションケア</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>3599</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210932470</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1198423707</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ポリジェン シークニング スカルプ コンディショニングマスク 200ml / 頭皮ケア ボリュームアップケア ハリコシ ダメージケア 保湿 しっとり サロンケア ヘアパック スカルプパック</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>3296</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198423707</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1196826611</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml / 保湿乳液 敏感肌対応 うるおいケア スキンケアローション 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G27" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196826611</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1164705875</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ウォータープルーフプロ日焼け止め 50g+サンスティック 20g / アウトドア スポーツ対応UVクリーム 汗・水に強いスティックタイプ 手を汚さない</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>5499</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164705875</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1207091316</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>manmulsang</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>レチノールスーパーバウンスセラム 20ml＋15ml 企画セット 初めてのレチノールケア 昼夜使いやすい 美容液 メイク前 なめらか肌印象 韓国コスメ スポイトタイプ 水分感 クリーム前 スキンケア</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>5324</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091316</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1185652076</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>bestkr</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>エリクシールウルティム オリジナルヘアオイル 30ml 1個 艶髪ケア うるおい 洗い流さないトリートメント サロン品質 ヘアケア デイリーケア 人気 コスパ 話題 限定 定番 口コミ多数 おすすめ</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ケラスターゼ</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>7140</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185652076</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1211858497</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NAVODA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>[大容量2個組] リジュラン トナーパッド ポアタイトニング つめかえ用 60枚入り 2個セット 毛穴 ピーリング 角質 スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211858497</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1204842932</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>NAVODA</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>[本品+リフィル] リジュラン ポア タイトニング トナーパッド 60枚+60枚 (計120枚) PDRN 毛穴ケア 弾력 ターンオーバー ダブル企画 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204842932</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1213317846</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>NAVODA</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>[送料無料] REJURAN リジュラン ダーマヒーラー ポアタイトニング ゲルマスク 2/3/4/5枚 毛穴ケア スキンケア 韓国コスメ シートマスク 保湿 弾력</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213317846</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1210050298</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NAVODA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>[送料無料/2本セット] ドクターフォーヘア エアロ クーリング スプレー 100ml / 頭皮ケア ドライシャンプー スカルプ 炭酸 冷却 ひんやり</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210050298</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J21"/>
+  <autoFilter ref="A1:J34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 12, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1849,8 +1849,541 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1178796694</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>[最新リニューアル] セルメディックス エムジーエフ リターンクリーム 70ml</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>cellmedics</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>8860</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178796694</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1180095461</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>イーロン アンプル 50ml センシエンド</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>15970</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095461</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1180095290</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>イーロン ダンギ クレンジングジェル 200ml + 贈呈:マスクパック1枚</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>6550</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095290</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1180095287</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ザ·イーロン イーロン メゾプロ プラスキット 1箱 2gx2個入 + スージング マスクパック 2枚</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>11880</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095287</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1180092834</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>サンテ 日焼け止め アズレン スーダー サンエッセンス 75ml 2個 デュオセット</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SANTE</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>15970</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180092834</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1191171558</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>sonny</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>[正規品] SKIN1004 プロバイオシカグロウサンアンプル, 50ml / SPF50+ PA++++ / 保湿 / スキンケア / 紫外線 / 乳液 / 白浮しない日焼け止め / オマケも /</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>2640</v>
+      </c>
+      <c r="G40" t="n">
+        <v>4</v>
+      </c>
+      <c r="H40" t="b">
+        <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191171558</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1097995675</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>kor_shop</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ルビーセル最新本物の保護マイルドラインミルク50ml強力で純粋なデイリーラインミルク50+</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Ruby-Cell</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>5826</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097995675</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1069605262</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>tovixkorea</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>セビウム エイチツーオー D 500ml（クレンジング+拭き取り化粧水）</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ビオデルマ</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>2390</v>
+      </c>
+      <c r="G42" t="n">
+        <v>3</v>
+      </c>
+      <c r="H42" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1069605262</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>1067966717</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>tovixkorea</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>[80枚/たっぷり310g] トナー 韓国コスメ 弱酸性 デイリー トナーパッド 角質ケア マスクシート 毛穴引き締め ハリ 弾力 肌キメ 水分 スキンケア トナー ピーリング ツヤ肌 コスメ</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NEEDLY</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>2740</v>
+      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1067966717</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1172740048</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tovixkorea</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Lactic Acid 5% + Hyaluronic Acid 2% Exfoliating Serum 30 ml</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>2380</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172740048</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>1172686121</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>tovixkorea</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Niacinamide 10% + Zinc 1% 30ml ナイアシンアミド10%+ジンク1%30ml</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1689</v>
+      </c>
+      <c r="G45" t="n">
+        <v>3</v>
+      </c>
+      <c r="H45" t="b">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172686121</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1162429093</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>yoo_k1120</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>コダリビノパーフェクトラジアンズセラム30mlホワイト ニングホワイト ニングアンプル（フランスセラム）</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>コーダリー</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>7340</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162429093</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1160701312</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>sweet_home</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>【追加料金なし】スウェットロールパッド 5枚入／顔汗対策／韓国製制汗シート／汗止めパッド</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" t="b">
+        <v>0</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160701312</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J34"/>
+  <autoFilter ref="A1:J47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 15, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2382,8 +2382,705 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1200996478</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>OSIO</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>スリーピング コパック カミング 10枚 大容量 / ブラックヘッド 毛穴 鎮静</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ケアプラス</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200996478</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1146775594</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>OSIO</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>【計100枚】緑豆 弱酸性 クレンジングティッシュ 20枚 x 5個</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>3330</v>
+      </c>
+      <c r="G49" t="n">
+        <v>3</v>
+      </c>
+      <c r="H49" t="b">
+        <v>0</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146775594</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1193530958</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>OSIO</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>【1+1】ポアシュリンカー バクチオールクリーム 60ml x 2個</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>マモンド</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>7560</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="b">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193530958</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>1152063267</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>OSIO</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>低刺激 フェイスアンド ボディ 大容量 日焼け止め 150mL (SPF50+ PA++++)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>シンムルナラ</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="b">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152063267</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1160024511</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SkinMuse</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ポテト マデカソサイド スージングパッド企画（60枚+60枚）水分パック/肌鎮静パック/低刺激</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>5400</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="b">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160024511</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1158858031</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SkinMuse</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>アトデルム シャワーオイル 1L 高保湿 敏感肌 乾燥肌 ボディウォッシュ フランスコスメ</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ビオデルマ</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>6200</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="b">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158858031</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1212491078</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SkinMuse</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Growturn Brush 130ml+30ml スカルプケア ヘアアンプル エクソソーム 頭皮ケア</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>5500</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="b">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212491078</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1204254720</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>k-pick72811</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>[ウォーターミストプランピング][正規品] マダガスカル センテラ ヒアル-テカ プランピング アンプル 50ml／スキンブースティング／ヒアルプラム</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>5743</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204254720</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1199087370</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>k-pick72811</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>[和解1位/脱毛シャンプー] パープルブースター [正規品]玉ねぎシャンプー/紫の抗酸化ブースター</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>prooted</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="b">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199087370</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>1206008183</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>247GOODLUCK</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ナイアシン トラネキサム酸13% セラム 30ml／トーンアップケア／肌荒れケア</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1565</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008183</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1203846979</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>247GOODLUCK</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>PDRN エアクラウド メラケア サンスクリーン 50ml #SPF50+ PA++++ #アルブチン #トラネクサン酸 #ナイアシンアミド #エラスチン #コラーゲン</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203846979</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1205520797</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ポアコントロール131 クレンジングオイル200ml／毛穴ケア／皮脂バランス</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>3153</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205520797</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1204558349</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>リポソームバブルブースター 95ml 2種（コラーゲン／キャビア PDRN）から1つ選択</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>3498</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204558349</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1118867909</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%エクスポリエイティングトナー 100ml韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>2346</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1118867909</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1188512361</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ノニアクネバブルクレンザー, 155ml /韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188512361</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1130886239</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>バイオガ ビオチン ダメージヘア改善 脱毛緩和シャンプー 1000ml /韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BIORGA</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130886239</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1097276457</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>リアルカレンデュラピールオフパック, 100g 韓国スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>3109</v>
+      </c>
+      <c r="G64" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097276457</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J47"/>
+  <autoFilter ref="A1:J64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 18, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3079,8 +3079,500 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1125939784</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>【正規品】グローアップインシャワートーンアップミルク300g</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>MEDIPICKME</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G65" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" t="b">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125939784</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1111189488</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>[単品] JunJun共同開発_クレンジングバーム2種 100ml (毛穴/トーンアップ)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="b">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1111189488</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1205453339</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>mellia</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ネックパッチプレステージ（5枚入り）首　シワ　弾力 ネックケア　アイロン　ハリケア 首のシワ 保湿 たるみ デコルテケア</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>VELLA</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205453339</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1125754461</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>[1+1]レッドブレミッシュクリアスージングクリーム 50ml 2個+10ml 2個/正規品</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>3469</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125754461</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1212553298</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>【正規品+GIFT付き】リードルショット コラーゲンクリーム 50ml＋スティックパウチ 3個</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>3021</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212553298</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1212350487</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>[1+1]MEDI AHAイボ取りクリーム25ml 2個&amp;nbsp; / メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>3666</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350487</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1212350471</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>[1+1]メディオルガブライトニングクリーム30ml 2個/しみ取りクリーム お肌のトーンアップ</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>3055</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350471</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1212350473</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>MEDI AHAイボ取りクリーム25ml/ メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350473</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1057808818</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>djshopping</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>LAB+トリプルウォーターピールスージングパッド 60枚</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>SNP</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>2390</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1057808818</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1205747267</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>アクニDr.ファーストブラックディープクレンジングフォーム 75ml</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>アイソイ</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>2286</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205747267</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1205745403</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>[6中1]練り香水 パフュームバーム 6.5g</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>5940</v>
+      </c>
+      <c r="G75" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205745403</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1205744981</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>シカカーミングパウダーウォッシュ 50g</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>TOCOBO</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205744981</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J64"/>
+  <autoFilter ref="A1:J76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 21, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3571,8 +3571,336 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1193630936</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>KTOPMARKET</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ガラク ナイアシン 3.0 エッセンス 60ml</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193630936</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1206871066</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>K_BrandPocket</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>タイムレボリューションレチノール500ショットラッピングマスク 1個 1個入り 集中パック ハリケア</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>2633</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206871066</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1191662969</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>bloomingseoul</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml(+ブルービーンクリーム7ml)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>2374</v>
+      </c>
+      <c r="G79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H79" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191662969</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1191657535</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>シカケア クリア アンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191657535</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1191655869</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>[新作]オールデイ ノーセバム トーンアップ サンクッション 2種 SPF45 PA++++ lilac fog vanilla lemon</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ミルクタッチ</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>3982</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191655869</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1188483946</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>キャロット カロテン デイリーマスク 30枚 #毎日使える栄養たっぷりのフェイスマスク</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>3777</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188483946</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1203329038</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>beauty69</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>【新作】スムース＆ピュア アイス クーリング デオ スプレー 150ml 2種</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>アリウル</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1581</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203329038</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1210434904</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>beauty69</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>[新作] NAD フリーズセル グロウブーストクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>5390</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210434904</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J76"/>
+  <autoFilter ref="A1:J84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 24, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3899,8 +3899,623 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1212154617</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>belif ビリーフ ザ・トゥルー クリーム モイスチャライジングバーム 50ml（保湿クリーム） (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ビリーフ</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>5170</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212154617</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1207926681</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>トリデン バランスフル シカ 鎮静クリーム 80ml(贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207926681</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1209840170</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>gmarketplus</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>クンダル プロテイン トリートメント イランイラン 500ml 3本 (贈呈品なくなり次第贈呈終了)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>5183</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209840170</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1060687901</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>gugumile</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Uriage ユリアージュ バリアダム シカクリーム 40ml [製造国 フランス]</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Uriage</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>3156</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="b">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1060687901</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1059767256</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>gugumile</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ROUND LAB ラウンドラップ 1025 独島 クレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1680</v>
+      </c>
+      <c r="G89" t="n">
+        <v>1</v>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1059767256</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1157418989</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>busanjin</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ゼロ毛穴 黒ずみ マッドパック 100g #AHA+BHA+PHA</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157418989</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1157419362</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>busanjin</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>[25SS/New]グリコリック アシッド 7% エクスポリエイティングトナー 240ml</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="b">
+        <v>0</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157419362</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1205905548</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>FROM051</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>メラレイジングアンプルクリーム 56g #シミケア #ナイアシンアミド #トラネキサム酸 #8種ヒアルロン酸</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>シャルド</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>5883</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="b">
+        <v>0</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205905548</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1210771223</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>PLUS82</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>マデカクリーム イン バブルセラム 100ml+100ml（+マデカパウダー ビタグルシ 6g）</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>6273</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="b">
+        <v>0</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210771223</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1206008325</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>ペプチドショット2X 弾力アンプル 30ml（ハリ感ケア／保湿／弾力サポート美容液）</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>2122</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008325</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1206008294</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ウォーターフィット リカバー BBクリーム 30ml #SPF40 PA+++ #保湿密着</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>2927</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008294</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1205912921</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>レチンアルブースターショット 30ml+30ml #レチナール2.0% #セラミド #エクトイン #カフェイン #ペプチド</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>4046</v>
+      </c>
+      <c r="G96" t="n">
+        <v>1</v>
+      </c>
+      <c r="H96" t="b">
+        <v>0</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205912921</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1209320737</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>[2PACK] クリーンイットゼロ 抹茶クレンジングバーム 100ml</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>4555</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" t="b">
+        <v>0</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209320737</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1201575924</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>[26SS/New]ピーチフェア ビーガン トーンアップ カプセルサンスクリーン 50ml #SPF50+ PA++++ #グルタチオン #ナイアシンアミド</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>ホイップド</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>3353</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="b">
+        <v>0</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201575924</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1201571343</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>[25SS/新作]4GF ザマ リペア ハイドロ セラム 30ml #エクソソーム #ナイアシンアミド #ペプチド #ノンコメドジェニック</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>CELORABY</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>5397</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="b">
+        <v>0</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201571343</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J84"/>
+  <autoFilter ref="A1:J99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 27, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J99"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4514,8 +4514,295 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1200699216</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>kbeautyroom88</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>(new)fuggler コラボ5種 コラーゲンペプチドジェリーセラムミスト/リジュビネイティングキャビア PDRN リアルディープマスク/ポアパーフェクティングコラーゲンペプチドセラム/リアルディー</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G100" t="n">
+        <v>3</v>
+      </c>
+      <c r="H100" t="b">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200699216</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1190875712</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>[26SS/New]セビウム セラム 30ml（+センシビオ H2O 5ml×2）</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>ビオデルマ</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>6600</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="b">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190875712</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1190240492</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>アップルタチオン トニング トナー パッド 60枚 #独自特許原料アップルタチオン #リンゴエキス+アロエ+高純度グルタチオン #鎮静</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>farmic</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>5168</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="b">
+        <v>0</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190240492</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1152717704</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>[26SS/New]ボディタミン アルファ ブライトニング スポット ボディセラム 80ml #ナイアシンアミド10%</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>ビヨンド</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>2948</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="b">
+        <v>0</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152717704</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1189199300</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>kurashiben</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>【18種類から自由に選べる】　ディーセス エルジューダ 全シリーズ 普通太い髪用 洗い流さないトリートメント メガ割 乳液 ヘアケア 美容室 サロン専売品 アウトバス ヘアパック ダメージケア</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>ミルボン</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1944</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="b">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189199300</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1212279783</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Poyo</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>【NEW】垢すり 角質ケア ソフトボディ レッドグローブ クリーン 1BOX (5枚入) 個包装 ボディスクラブ ボディクレンジング 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="b">
+        <v>0</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212279783</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1202082347</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>lindalinda</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>【垢すり/角質ケア】ソフトボディ レッドグローブ クリーン 1BOX(5枚入) / 個包装 / ボディクレンジング / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>ランドリーユー</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>2520</v>
+      </c>
+      <c r="G106" t="n">
+        <v>5</v>
+      </c>
+      <c r="H106" t="b">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202082347</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J99"/>
+  <autoFilter ref="A1:J106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 30, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4801,8 +4801,705 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1205730098</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>dsire88</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>[NEW]アトバリア 365 カプセルトナー 300ml/アトバリア/韓国スキンケア/PHA/カプセルトナー/セラミド/保湿/アトバリア 化粧水/乾燥肌/水分</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>3996</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="b">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205730098</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>1093447562</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>dsire88</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ーモイスチャートリトメントマスク 5枚/保湿ケア</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G108" t="n">
+        <v>1</v>
+      </c>
+      <c r="H108" t="b">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093447562</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1205513550</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>dsire88</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>[新商品発売]パンテノール リキッドエッセンス サンセラム SPF50+ PA+++, 50ml/ 軽やかに密着するウォーターセラムテクスチャー/クーリング/パンテノール2%/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>4585</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="b">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205513550</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1211478917</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>deesse1128</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>【26年新リニューアル】ダルバ ヴィーガン ヘアパフュームセラム 100ml ヘアミスト 保湿 ダメージケア 韓国コスメプロフェッショナルリペアリングヘアパフュームセラム</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="b">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211478917</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1213065508</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>deesse1128</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>【2026新作】ダルバ エアフィット ブルー トーンアップUVパウダー 5.5g SPF UVケア 毛穴カバー テカリケア ヴィーガン</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" t="b">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213065508</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1205554324</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>deesse1128</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>[NEW][ダルバ ウォータフル パンテノール UVセラム 50ml クーリング 水分UV 低刺激 ヴィーガン 敏感肌 韓国コスメ SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G112" t="n">
+        <v>3</v>
+      </c>
+      <c r="H112" t="b">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205554324</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1209315395</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>deesse1128</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>息をするような軽さ雲のような密着感エアクラウド ウォーターパウダー サンクッション 01 ブルー/ベースメイク/崩れにくい/サラサラ肌</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="b">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209315395</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1195790484</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>UNICOSMETIC</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>【限定15%OFF】イロン ダンギ スージングジェル 500ml 韓国コスメ l マルチジェル l うるおいケア l さっぱりとしたテクスチャー l 熱感ケア</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>7990</v>
+      </c>
+      <c r="G114" t="n">
+        <v>4</v>
+      </c>
+      <c r="H114" t="b">
+        <v>0</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195790484</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1196819316</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>ktrendmall</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>グルタチオンビタシートマスク デイリーピック 30枚</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>2734</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="b">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196819316</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1182043662</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>ktrendmall</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>エクソソームシカ ツボクサ鎮静クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="b">
+        <v>0</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182043662</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1190079671</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>dailyozzi</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】（リニューアル）エイシカ365 スージングリペアクリームpH4.5 60ml +【セラム 7ml+パッド5ml 2枚】べたつかない保湿肌ダーマコスメティック</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>2889</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="b">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190079671</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1164572795</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>dailyozzi</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>【NEW】ディープクレンジングオイル225ml+クレンジングオイル25ml+クレンジングフォーム 15g+メイク落とし 15ml /毛穴ケア/保湿効果</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>ヘラ</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>4761</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" t="b">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164572795</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1193548089</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>dailyozzi</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】NewダーマUV日焼け止め 40ml UV カット【+日焼け止め20ml贈呈】セラミド ヒアルロン酸配合／保湿チャージ／ビタC</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>2961</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="b">
+        <v>0</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193548089</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1206682479</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>cafebespoke</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>グリーンプロポリス 頭皮クレンジング シャンプー+トリートメント [1000ml+1000ml] セット</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G120" t="n">
+        <v>3</v>
+      </c>
+      <c r="H120" t="b">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206682479</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>1206870778</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>mood_k</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>345 リリーフ クリームミスト 100ml+60ml 保湿ミスト 韓国コスメ 敏感肌 乾燥対策 フェイスミスト スキンケア</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>4240</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="b">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206870778</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>1209089569</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>mokos_kshop</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>the SAEM アーバンエコ ハラケケ トナー 150ml1個 韓国化粧水 高保湿 乾燥肌 敏感肌 スキンケア 水分補給 保湿トナー</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="b">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089569</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>1209089497</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>mokos_kshop</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>the SAEM アーバンエコ ハラケケ トナー 150ml 2個 set/韓国化粧水 高保湿 乾燥肌 敏感肌 スキンケア 水分補給 保湿トナー</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="b">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209089497</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J106"/>
+  <autoFilter ref="A1:J123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 33, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J123"/>
+  <dimension ref="A1:J131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5498,8 +5498,336 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>1156030393</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>3番 ノーファンデ陶器肌トーンアップクリーム 50ml (2個)</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>7120</v>
+      </c>
+      <c r="G124" t="n">
+        <v>1</v>
+      </c>
+      <c r="H124" t="b">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156030393</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>1188366439</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>[NEW] [新商品] 9番 NMN PDRN グロー トリートメント トナー 150ml (2個)</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>6573</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="b">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188366439</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>1180595613</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>PDRN 100ヒアルロン酸 ブースター トナー 250ml + PDRNヒアルロン酸100モイスチャライジングクリーム 60ml + PDRN ヒアルロン酸カプセル 100セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>11931</v>
+      </c>
+      <c r="G126" t="n">
+        <v>1</v>
+      </c>
+      <c r="H126" t="b">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180595613</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>1180594432</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>[NEW] [新商品] PDRN 100ヒアルロン酸 ブースター トナー 250ml (2個) + PDRN ヒアルロン酸カプセル 100セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>11061</v>
+      </c>
+      <c r="G127" t="n">
+        <v>1</v>
+      </c>
+      <c r="H127" t="b">
+        <v>0</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180594432</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>1180589025</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>[NEW] [新商品] ドクダミ 77 スージングトナー 250ml + ドクダミ 70 デイリー ローション 200ml + ドクダミポアコントロールクレンジングオイル 200ml (2個)</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>12056</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="b">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180589025</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1163571137</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>K-BEAUTYBOX</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>グッセラスーパーセラミドクリーム 60ml 2個 高保湿クリームナイトケア</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>ホリカホリカ</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>4584</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="b">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163571137</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>1168069878</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>morningmood</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>白樺 水分トナー 300ml</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>2345</v>
+      </c>
+      <c r="G130" t="n">
+        <v>1</v>
+      </c>
+      <c r="H130" t="b">
+        <v>0</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168069878</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>1176812478</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>meisonmatcha</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>[2個]トータルリペア5 ミラクル ヘアパック 170ml</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>1626</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="b">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176812478</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J123"/>
+  <autoFilter ref="A1:J131"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 36, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$153</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J131"/>
+  <dimension ref="A1:J153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5826,8 +5826,910 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>1205779441</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>albami</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>エストラ アトバリア365 ハイドロ スージングクリーム 80ml セット(トナー25ml+クレンジングフォーム30g)</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>ハイドロ</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>4450</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="b">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205779441</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1204919251</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>bluepearl</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>【リニューアル】アトバリア365ハイドロスージングクリーム, 80ml</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>3554</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" t="b">
+        <v>0</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204919251</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1202057017</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>bluepearl</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>【NEW】ザブルーペプチドセラム, 50ml</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>3250</v>
+      </c>
+      <c r="G134" t="n">
+        <v>1</v>
+      </c>
+      <c r="H134" t="b">
+        <v>0</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202057017</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>1194043789</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>bluepearl</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>RXザビタミンC23セラム2世代, 20g, 2個</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>4885</v>
+      </c>
+      <c r="G135" t="n">
+        <v>4</v>
+      </c>
+      <c r="H135" t="b">
+        <v>0</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194043789</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>1179722209</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>bluepearl</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>ザモイスチャーバリアDリキッドトナー, 200ml</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G136" t="n">
+        <v>3</v>
+      </c>
+      <c r="H136" t="b">
+        <v>0</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179722209</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>1213443102</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>[正規品]アーバンエコ ハラケケ トナー 150ml, 1個</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>3028</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" t="b">
+        <v>0</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213443102</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>1200735680</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>[正規品]ALL NEW シグニア リファイニング ウォーターエッセンス 180ml, 1個</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>ヘラ</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>10543</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" t="b">
+        <v>0</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200735680</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>1196714483</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>[正規品] レチノール レティジェクション セラム 30ml, 1個</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>7345</v>
+      </c>
+      <c r="G139" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" t="b">
+        <v>0</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196714483</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>1165247523</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>[正規品] オールデイ メイクアップフィクサー 75ml 1個</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>3013</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="b">
+        <v>0</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165247523</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>1213167963</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>[正規品]インテンスケア ゴールド 24K スネイルフォームクレンザー 150ml, 1個</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>2434</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" t="b">
+        <v>0</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213167963</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>1213378280</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>ザ・ビタA レチナールショット タイトニングブースター 15ml/더 비타 A 레티날 샷 타이트닝 부스터 15ml</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>2386</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" t="b">
+        <v>0</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213378280</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>1167189215</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>ドクダミヒアルロンスージング アンプル 50ml/ 어성초 히알루론 수딩 앰플 50ml</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>2212</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" t="b">
+        <v>0</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167189215</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>1083286884</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BB_KO</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>[ エンジェルスリキッド ] グルタチオンプラス ナイアシンアミド 700vクリーム 50ml/나이아신아마이드 700v 크림</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Angel's Liquid</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>3085</v>
+      </c>
+      <c r="G144" t="n">
+        <v>3</v>
+      </c>
+      <c r="H144" t="b">
+        <v>0</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083286884</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>1211694332</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>blanc-lapin</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>ジュリーク JURLIQUE RO バランシングミスト 100ml 化粧水 [169628]</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>ジュリーク</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>4460</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="b">
+        <v>0</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211694332</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>1205909859</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>blanc-lapin</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>【本体フィルム剥がれあり】クラランス CLARINS グランアイセラムV 15ml [448368]</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>クラランス</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>5580</v>
+      </c>
+      <c r="G146" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" t="b">
+        <v>0</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205909859</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>1181847777</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>【ポムポムプリンコラボ】ライティングトーンアップサンクッション/ヴィーガンリリーフサンクリーム/サンエッセンス/オーセンティックリップグロイバーム/セット企画 / オリーブヤング限定</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>アッテ</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G147" t="n">
+        <v>2</v>
+      </c>
+      <c r="H147" t="b">
+        <v>0</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181847777</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>1213323194</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>【ピングーコラボ】全種まとめ ポストアルファクーリングパッド 70枚+70枚 / クーリングペプチドアンプル 30ml / ファーストクーリングマスク 5+3枚 / シカクーリングマスク 5+3枚</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>2310</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" t="b">
+        <v>0</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213323194</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>1201547339</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>パフュームハンドクリーム [ハローキティ], 50ml</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>ヘトラス</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>2170</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" t="b">
+        <v>0</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201547339</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>1172312020</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>hokkorikorea</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>【SALE】【毛穴ケア】PDRN毛穴弾力パッド 100枚 ハリ感 キメ整う エイジングケア ツヤ肌 角質ケア うるおい 人気 韓国コスメ 大容量 毎日ケア 時短 敏感肌OK 透明感 キメケア 保湿</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>3006</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" t="b">
+        <v>0</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172312020</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>1211709109</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>leoshopkorea</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>ミジャンセン サロン10 タンパク質 トリートメント 280ml ハイダメージ 髪質改善 補修 保湿 ヘアケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>2541</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="b">
+        <v>0</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211709109</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>1196218945</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>leoshopkorea</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>[薬局専用]リジュブースター Rejuvuster PDRN リジュビネイティングクリーム 25ml / 韓国薬局専用 高濃度サーモンDNA 集中ケア 肌バリア 正規品</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>PYDERIN</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>4902</v>
+      </c>
+      <c r="G152" t="n">
+        <v>4</v>
+      </c>
+      <c r="H152" t="b">
+        <v>0</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196218945</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>1195464780</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>leoshopkorea</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>[1+1]大容量 メラトーニング ワンデーアンプル 30ml +30ml 大容量 / 韓国NO.1シミケアアンプル DW-EGF配合 コスパ 肝斑 そばかす 集中ケア 正規品</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>イージーデュー</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>11891</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="b">
+        <v>0</v>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195464780</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J131"/>
+  <autoFilter ref="A1:J153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 39, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J153"/>
+  <dimension ref="A1:J164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6728,8 +6728,459 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>1183055576</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Asteroid</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>シャンプー ダマスクローズの香り 1L</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>ミルクバオバブ</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>2745</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="b">
+        <v>0</v>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183055576</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>1133994465</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Asteroid</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>24K ラグジュアリー ゴールド アンプル 110ml</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>BERGAMO</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>3813</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="b">
+        <v>0</v>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133994465</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>1204446765</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>SarangCosme</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>クーリングサンスプレー SPF50+ PA+++ 150ml</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>ドクターアト</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="b">
+        <v>0</v>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204446765</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>1187961675</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>SarangCosme</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>[アイメイク防水] メイクアップ セッティング マルチ マジック シーラー フィクサー 10ml</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>1805</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="b">
+        <v>0</v>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187961675</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>1195129454</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>K_AUTHENTIC</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>[韓國正品店]NEW Love portion オードパルファム 香水 9種/韓国人氣</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>After blow</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="b">
+        <v>0</v>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195129454</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>1150649094</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>tiaramall</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>[1+1]センテラ クイックカーミングパッド 70枚入り2個/パックパッドトナーパッド化粧水トナー鎮静水分保湿</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>3591</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="b">
+        <v>0</v>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150649094</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>1182384650</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>hanbikosupa</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>マスクフィット メイクアップ クールフィクサー 80ml 韓国コスメ メイクキープスプレー</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>2680</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="b">
+        <v>0</v>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182384650</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>1196852846</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>AC ディープカミング ポア サンスティック 20g x 1個 / SPF 50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>デューイーツリー</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="b">
+        <v>0</v>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196852846</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>1132737248</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>バランシウム セラミド 高保湿シート マスク 26ml x 10枚</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>3960</v>
+      </c>
+      <c r="G162" t="n">
+        <v>2</v>
+      </c>
+      <c r="H162" t="b">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132737248</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>1130447122</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>3番 結果いっぱいのエッセンス トナー 200ml (50種類の発酵/肌の輝き/弾力)</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" t="b">
+        <v>0</v>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130447122</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>1209269112</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>【1+1】マデカソサイド保湿サンスリーム 痕跡リペア 50+50g / SPF 50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>4320</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="b">
+        <v>0</v>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209269112</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J153"/>
+  <autoFilter ref="A1:J164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 42, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$175</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J164"/>
+  <dimension ref="A1:J175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7179,8 +7179,459 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>1163367685</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>leeleeshop</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>[NEW]レッド アクネ ボディピーリングショット 110g</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G165" t="n">
+        <v>1</v>
+      </c>
+      <c r="H165" t="b">
+        <v>0</v>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163367685</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>1206889838</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>leeleeshop</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>スーディング プリップ リップマスク</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Laka</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>2448</v>
+      </c>
+      <c r="G166" t="n">
+        <v>1</v>
+      </c>
+      <c r="H166" t="b">
+        <v>0</v>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206889838</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>1106986645</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>TeaTime</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>【2個セット】シークレット マルチバーム 7g×2 発酵保湿スティック 韓国コスメ 携帯用 高保湿 ツヤ肌 ハリケア</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>4399</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="b">
+        <v>0</v>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1106986645</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>1201560856</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>[NEW] PDRN カフェイン 1000 オーバーナイト ラッピング マスク 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>P.CALM</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>4100</v>
+      </c>
+      <c r="G168" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" t="b">
+        <v>0</v>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201560856</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>1208992240</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>[NEW] マイルド ヴィーガン トーンアップ 日焼け止め 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G169" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" t="b">
+        <v>0</v>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208992240</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>1191141866</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>[NEW] スーパー コラーゲン バブル セラム マスク 90g 1個</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>AROCELL</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>5550</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="b">
+        <v>0</v>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191141866</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>1168717728</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>[新商品] キャロット カロチン モイスト エフェクター 55ml 1個</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" t="b">
+        <v>0</v>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168717728</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>1146804177</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>fourheart</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>[正品] ゼロ 毛穴 ブラックヘッド ディープ クレンジングオイル 205ml 1個</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" t="b">
+        <v>0</v>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146804177</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>1181843699</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>k-sunshop</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>ステム3 クリーム 5ml x 10個</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G173" t="n">
+        <v>1</v>
+      </c>
+      <c r="H173" t="b">
+        <v>0</v>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181843699</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>1181410808</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>k-sunshop</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>ハイアルロン エピセリンセラム 30ml</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>ユーセリン</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>5400</v>
+      </c>
+      <c r="G174" t="n">
+        <v>2</v>
+      </c>
+      <c r="H174" t="b">
+        <v>0</v>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181410808</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>1107510664</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>KSB</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>[新作]ムード レイヤー スティック クレヨン 5color 00 milky syrup 01 caramel drizzle 02 rose milk tea 03 mauve latte</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>alternative stereo</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>2405</v>
+      </c>
+      <c r="G175" t="n">
+        <v>1</v>
+      </c>
+      <c r="H175" t="b">
+        <v>0</v>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1107510664</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J164"/>
+  <autoFilter ref="A1:J175"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 45, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$181</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J175"/>
+  <dimension ref="A1:J181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7630,8 +7630,254 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>1212102383</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>SUGARJELLY</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>ミラクル2X ヘアトリートメント ネロリの香り 180ml / ネロリフラワー / ダメージケア・集中保湿 / サロン品質 / 洗い流さないトリートメント / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>モレモ</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>1665</v>
+      </c>
+      <c r="G176" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" t="b">
+        <v>0</v>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212102383</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>1205142771</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>SUGARJELLY</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>マルチペプチドセラム フォー ヘア デンシティ 30ml / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>2902</v>
+      </c>
+      <c r="G177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H177" t="b">
+        <v>0</v>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205142771</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>1210577063</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>wingkone</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>【正規品】【NEW】【脱色/染め】 眉毛脱色 イージーブロウトーンチェンジャー 5回分 / イージーブロウムードチェンジャー 5回分 / アイブロウ / 韓国コスメ / 眉毛</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G178" t="n">
+        <v>3</v>
+      </c>
+      <c r="H178" t="b">
+        <v>0</v>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210577063</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>1209903581</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>【ニキビケア】[1+1]1番 パントテン酸アクティブスージングクリーム 80ml/ニキビ</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G179" t="n">
+        <v>0</v>
+      </c>
+      <c r="H179" t="b">
+        <v>0</v>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209903581</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>1198095545</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>【GIFT】洗顔/ゼロ 毛穴 ブラックヘッド ディープ クレンジングオイル 205ml/毛穴ケア/毛穴 黒ずみ/ブラックヘッド/韓国コスメ 毛穴</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G180" t="n">
+        <v>0</v>
+      </c>
+      <c r="H180" t="b">
+        <v>0</v>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198095545</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>1110469138</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>【5種沢1】CICA/PDRN/毛穴/ニキビケア/保湿／トナーパット／鎮静／トナー／化粧水/毛穴ケア/ふき取り化粧水/メが割/美容液</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>2995</v>
+      </c>
+      <c r="G181" t="n">
+        <v>0</v>
+      </c>
+      <c r="H181" t="b">
+        <v>0</v>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110469138</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J175"/>
+  <autoFilter ref="A1:J181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 48, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$194</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J181"/>
+  <dimension ref="A1:J194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7876,8 +7876,541 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>1116944837</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>dal25</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>9種の中から 選択1 / ゴールドコアマックスキッズ肝臓ケア植物性糖ケアスリム50代 韓国製品 韓国乳酸菌 乳酸菌 キッズ プロバイオティクス ミルクシスル ガルシニア ビタミンD 生乳酸菌</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>ラクトフィット</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>2580</v>
+      </c>
+      <c r="G182" t="n">
+        <v>5</v>
+      </c>
+      <c r="H182" t="b">
+        <v>0</v>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1116944837</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>1115638534</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>dal25</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>旅行用ヘアボディ5種+コットンポーチ1セット 韓国シャンプー 純正品 旅行キット トラベルキット トリートメント ボディウォッシュ ボディローション クレンジングフォーム 旅行 携帯用シャンプー</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>NARD</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G183" t="n">
+        <v>0</v>
+      </c>
+      <c r="H183" t="b">
+        <v>0</v>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115638534</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>1123888012</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>unopick</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>リードルショット1000 エッセンス 15ml</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>5700</v>
+      </c>
+      <c r="G184" t="n">
+        <v>1</v>
+      </c>
+      <c r="H184" t="b">
+        <v>0</v>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123888012</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>1123548274</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>unopick</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド 10 TXA 4 ダークスポット コレクティング セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>4940</v>
+      </c>
+      <c r="G185" t="n">
+        <v>0</v>
+      </c>
+      <c r="H185" t="b">
+        <v>0</v>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123548274</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>1147146315</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>jinytrading</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>PDRN ピンク グルタチオン セラム ミスト 100ml 水分 保湿 弾力 韓国化粧品 韓国美容ギフト</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>2961</v>
+      </c>
+      <c r="G186" t="n">
+        <v>0</v>
+      </c>
+      <c r="H186" t="b">
+        <v>0</v>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147146315</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>1159784308</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>jinytrading</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>ビタCプラス アスコルビン酸 クリアコンプレクション フォーミングクレンザー 120ml 高濃度ビタミンC フォームクレンジング 水分 保湿 韓国化粧品 韓国美容ギフト</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>1971</v>
+      </c>
+      <c r="G187" t="n">
+        <v>0</v>
+      </c>
+      <c r="H187" t="b">
+        <v>0</v>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159784308</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>1205563457</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>ガラクトミー エンザイム ピーリングジェル, 75ml, 1個</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>1829</v>
+      </c>
+      <c r="G188" t="n">
+        <v>0</v>
+      </c>
+      <c r="H188" t="b">
+        <v>0</v>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205563457</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>1171042034</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>アクティブクリーンアップクレンジングパウダー酵素洗顔剤, 80g</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>4005</v>
+      </c>
+      <c r="G189" t="n">
+        <v>1</v>
+      </c>
+      <c r="H189" t="b">
+        <v>0</v>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171042034</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>1188510609</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>AVECPUBLIC</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>スーパージェクションクリーム, 20ml</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>7560</v>
+      </c>
+      <c r="G190" t="n">
+        <v>3</v>
+      </c>
+      <c r="H190" t="b">
+        <v>0</v>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188510609</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>1164282563</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>GlowMG</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>プロテクション マイルド サンミルク 50ml (2個)</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Ruby-Cell</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>7379</v>
+      </c>
+      <c r="G191" t="n">
+        <v>1</v>
+      </c>
+      <c r="H191" t="b">
+        <v>0</v>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164282563</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>1135274021</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>GlowMG</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>ロックセント ボディローション 488ml / 4種 1択 / ヒノキ / グリーンローズ / ベルガモット / アースフィグ</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>MARMAR;D</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>2137</v>
+      </c>
+      <c r="G192" t="n">
+        <v>2</v>
+      </c>
+      <c r="H192" t="b">
+        <v>0</v>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135274021</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>1135414332</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>calluna</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>[ギフト包装] ミスト セラム 100ml + ハンドクリーム 30ml + 鏡</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>3934</v>
+      </c>
+      <c r="G193" t="n">
+        <v>2</v>
+      </c>
+      <c r="H193" t="b">
+        <v>0</v>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135414332</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>1170532806</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>calluna</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>【ポムポムプリン限定企画】ビーガンパックレンザー3種択1 (グリーントマト120ml/ レッドトマト120ml/ ライスドウ130ml)</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>FULLY</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>2525</v>
+      </c>
+      <c r="G194" t="n">
+        <v>3</v>
+      </c>
+      <c r="H194" t="b">
+        <v>0</v>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170532806</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J181"/>
+  <autoFilter ref="A1:J194"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 51, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$199</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J194"/>
+  <dimension ref="A1:J199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8409,8 +8409,213 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>977992270</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>farfallarossa</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>パナソニック リフトケア 美顔器 バイタリフト かっさ 温感 デュアルダイナミックEMS搭載 防水</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>パナソニック</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>33208</v>
+      </c>
+      <c r="G195" t="n">
+        <v>1</v>
+      </c>
+      <c r="H195" t="b">
+        <v>0</v>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=977992270</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>1205052684</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>MOMOCHI_SHOP</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>【毛穴洗顔】 ゼロ毛穴 クレンジングフォーム 120g サリチル酸 BHA洗顔 カプセル洗顔 韓国洗顔 毛穴ケア 皮脂ケア フォーム洗顔 韓国スキンケア 角質ケア 毛穴汚れ 韓国コスメ デイリー洗顔</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G196" t="n">
+        <v>0</v>
+      </c>
+      <c r="H196" t="b">
+        <v>0</v>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205052684</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>1212968157</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>MOMOCHI_SHOP</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>【目元ハリケア】 アイファルト アイバック クリーム 10ml 目元たるみ アイクリーム 保湿 レチノール EGF ナイアシンアミド セラミド 目元ケア 乾燥小じわ 韓国コスメ くまケア</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G197" t="n">
+        <v>0</v>
+      </c>
+      <c r="H197" t="b">
+        <v>0</v>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212968157</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>1206857284</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>k_town</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>【正規品】コンブチャミスト 100ml + 選べるプレゼント / スペシャルケアマスクパック</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>エリシャコイ</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>2123</v>
+      </c>
+      <c r="G198" t="n">
+        <v>0</v>
+      </c>
+      <c r="H198" t="b">
+        <v>0</v>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206857284</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>1138225289</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>dreamus</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>シグネチャーパルファム, 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>5517</v>
+      </c>
+      <c r="G199" t="n">
+        <v>0</v>
+      </c>
+      <c r="H199" t="b">
+        <v>0</v>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138225289</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J194"/>
+  <autoFilter ref="A1:J199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 54, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$209</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J199"/>
+  <dimension ref="A1:J209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8614,8 +8614,418 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>1109209881</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>korkorshop</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>[NEW]ヒストラップイージーエフコンプレックスアンプル63％80ml / EGF</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>HISTOLAB</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>9737</v>
+      </c>
+      <c r="G200" t="n">
+        <v>0</v>
+      </c>
+      <c r="H200" t="b">
+        <v>0</v>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109209881</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>1211721947</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>ポアタイトニング クレンジングバーム 50ml × 2個セット</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>7482</v>
+      </c>
+      <c r="G201" t="n">
+        <v>0</v>
+      </c>
+      <c r="H201" t="b">
+        <v>0</v>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211721947</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>1137919225</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>パンテノール クリームウォッシュ 300ml × 2本</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>6253</v>
+      </c>
+      <c r="G202" t="n">
+        <v>0</v>
+      </c>
+      <c r="H202" t="b">
+        <v>0</v>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137919225</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>1211388494</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>ウォーターカプセル サンセラム SPF50+ / PA+++ 40ml × 2個セット</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>7482</v>
+      </c>
+      <c r="G203" t="n">
+        <v>0</v>
+      </c>
+      <c r="H203" t="b">
+        <v>0</v>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211388494</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>1205514714</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Nandak</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>[ダーママスク10枚プレゼント] マデカクリームハイドラカーミング50ml3個韓国人気化粧品</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>5850</v>
+      </c>
+      <c r="G204" t="n">
+        <v>1</v>
+      </c>
+      <c r="H204" t="b">
+        <v>0</v>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205514714</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>1080770379</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>NARShA</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>ライトオンインシャワーボディトーンアップボディローション ベビーパウダーの香り290ml</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>4720</v>
+      </c>
+      <c r="G205" t="n">
+        <v>0</v>
+      </c>
+      <c r="H205" t="b">
+        <v>0</v>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080770379</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>1206876054</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>NARShA</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>[ブラシ元祖] グロウターンエクソソームブラシアンプル130ml企画(+30ml)</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F206" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G206" t="n">
+        <v>0</v>
+      </c>
+      <c r="H206" t="b">
+        <v>0</v>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206876054</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>1204156842</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>[1+1] トン＆スポット コレクターアンプル 30ml +30ml</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Redence</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G207" t="n">
+        <v>2</v>
+      </c>
+      <c r="H207" t="b">
+        <v>0</v>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204156842</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>1186174034</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>[1+1]アルガンオイルダメージトリートメント300ml+300ml</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>エラスティン</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G208" t="n">
+        <v>0</v>
+      </c>
+      <c r="H208" t="b">
+        <v>0</v>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186174034</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>1156719535</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>ソウルシークレットブロッサム香水30ml</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>ザフェイスショップ</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G209" t="n">
+        <v>0</v>
+      </c>
+      <c r="H209" t="b">
+        <v>0</v>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156719535</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J199"/>
+  <autoFilter ref="A1:J209"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 57, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$209</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$221</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J209"/>
+  <dimension ref="A1:J221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9024,8 +9024,500 @@
         </is>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>1080682873</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>momonara</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>ザ ヒアルロニック アシード 3 セラム 20ml</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F210" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G210" t="n">
+        <v>0</v>
+      </c>
+      <c r="H210" t="b">
+        <v>0</v>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080682873</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>1079892554</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>momonara</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>ピュアフィット シカ カーミング トゥルーシートマスク 10枚</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G211" t="n">
+        <v>0</v>
+      </c>
+      <c r="H211" t="b">
+        <v>0</v>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1079892554</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>1205346742</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>KKK-Shop</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>[メガ割] TAMBURIN*S タンバリン*ズ ヘアオイル 50ml サマーテイルズ イブニンググロウ カモ ダメージ補修 ツヤ 潤い 香り 髪質改善 スタイリング フレグランス 韓国ヘアケア 正規</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>5481</v>
+      </c>
+      <c r="G212" t="n">
+        <v>0</v>
+      </c>
+      <c r="H212" t="b">
+        <v>0</v>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205346742</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>1194293129</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>hancony</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド20 セラム 40ml</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>JUMISO</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G213" t="n">
+        <v>0</v>
+      </c>
+      <c r="H213" t="b">
+        <v>0</v>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194293129</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>1153497615</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Vividgrow</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>AHA 30% + BHA 2% ピーリングソリューション 30ml</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F214" t="n">
+        <v>2597</v>
+      </c>
+      <c r="G214" t="n">
+        <v>0</v>
+      </c>
+      <c r="H214" t="b">
+        <v>0</v>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1153497615</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>1152849853</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Vividgrow</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>[26SS/New]デオキシリボス 頭皮強化アンプル 20ml #エクソソーム #ビオチン #EGF</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>4652</v>
+      </c>
+      <c r="G215" t="n">
+        <v>0</v>
+      </c>
+      <c r="H215" t="b">
+        <v>0</v>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152849853</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>1171460964</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Vividgrow</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>パフュームドポ ボディウォッシュ 600ml 2種から1つ選択</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>VEILMENT</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>2532</v>
+      </c>
+      <c r="G216" t="n">
+        <v>0</v>
+      </c>
+      <c r="H216" t="b">
+        <v>0</v>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171460964</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>1166654877</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Vividgrow</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>[26SS/New]アイパッチ 60枚 2種（コラーゲン／キャビア PDRN）から1つ選択</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>2851</v>
+      </c>
+      <c r="G217" t="n">
+        <v>0</v>
+      </c>
+      <c r="H217" t="b">
+        <v>0</v>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1166654877</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>1109964483</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Beauty-Life</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>ハイドラローションマックス 400ml</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>エステダム</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>8125</v>
+      </c>
+      <c r="G218" t="n">
+        <v>0</v>
+      </c>
+      <c r="H218" t="b">
+        <v>0</v>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109964483</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>1109951025</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Beauty-Life</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>シアーシュガー スクラブ 510g 11種 ビタミンC</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Tree Hut</t>
+        </is>
+      </c>
+      <c r="F219" t="n">
+        <v>4225</v>
+      </c>
+      <c r="G219" t="n">
+        <v>0</v>
+      </c>
+      <c r="H219" t="b">
+        <v>0</v>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109951025</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>1200859567</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>ALLROUNDERBEAUTY</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>ティーツリーシカ ディープクレンジングオイル 200ml</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F220" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G220" t="n">
+        <v>0</v>
+      </c>
+      <c r="H220" t="b">
+        <v>0</v>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200859567</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>1162838579</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>tmashop</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>[単独企画]清楚ビタCジョブティケアパッド70枚（10枚贈呈）</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F221" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G221" t="n">
+        <v>0</v>
+      </c>
+      <c r="H221" t="b">
+        <v>0</v>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162838579</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J209"/>
+  <autoFilter ref="A1:J221"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 60, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$239</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J221"/>
+  <dimension ref="A1:J239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9516,8 +9516,746 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>1180348089</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>SOFS</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>シークレットエッセンス 45ml しっとり肌</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F222" t="n">
+        <v>3121</v>
+      </c>
+      <c r="G222" t="n">
+        <v>0</v>
+      </c>
+      <c r="H222" t="b">
+        <v>0</v>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180348089</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>1203096775</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>SOFS</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>フィディアルエン(PDRN)毛穴タイトニングパッド(100pcs) リフティング</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F223" t="n">
+        <v>2691</v>
+      </c>
+      <c r="G223" t="n">
+        <v>0</v>
+      </c>
+      <c r="H223" t="b">
+        <v>0</v>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203096775</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>1180349223</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>SOFS</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>マデカセンテラスーディングミスト100ml ツボクサ 鎮静スプレー</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F224" t="n">
+        <v>2597</v>
+      </c>
+      <c r="G224" t="n">
+        <v>1</v>
+      </c>
+      <c r="H224" t="b">
+        <v>0</v>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180349223</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>1180349101</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>SOFS</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>エッセンスミスト 60ml+60ml SET</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>3392</v>
+      </c>
+      <c r="G225" t="n">
+        <v>0</v>
+      </c>
+      <c r="H225" t="b">
+        <v>0</v>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180349101</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>1180349080</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>SOFS</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>シルクヘアリペアオイル130ml</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>1969</v>
+      </c>
+      <c r="G226" t="n">
+        <v>1</v>
+      </c>
+      <c r="H226" t="b">
+        <v>0</v>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180349080</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>1208195309</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>klumin</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>パフュームシルキーハンドクリーム50ml フレグランス12種, ご購入でMEDIHEAL ローズPDRNマスク1枚プレゼント</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>ヘトラス</t>
+        </is>
+      </c>
+      <c r="F227" t="n">
+        <v>1940</v>
+      </c>
+      <c r="G227" t="n">
+        <v>0</v>
+      </c>
+      <c r="H227" t="b">
+        <v>0</v>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208195309</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>1209668463</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>klumin</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>[MEDIHEAL マスク1枚付き]ドクダミ77スージングトナー，350ml</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F228" t="n">
+        <v>2926</v>
+      </c>
+      <c r="G228" t="n">
+        <v>0</v>
+      </c>
+      <c r="H228" t="b">
+        <v>0</v>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209668463</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>1208085435</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>[26SS/New]クリアライスサンスクリーン 50ml（+20ml＋チュンシキキーホルダー）</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F229" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G229" t="n">
+        <v>0</v>
+      </c>
+      <c r="H229" t="b">
+        <v>0</v>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208085435</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>1208085817</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>(ポケモンエディション)体臭ソリューション デオドラント ボディウォッシュ 720ml 2種から1つ選択</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>46CM</t>
+        </is>
+      </c>
+      <c r="F230" t="n">
+        <v>2889</v>
+      </c>
+      <c r="G230" t="n">
+        <v>0</v>
+      </c>
+      <c r="H230" t="b">
+        <v>0</v>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208085817</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>1199735232</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>VividgrowMAN</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>PDRNピンクエクソソームショット2000, 30ml</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F231" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G231" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" t="b">
+        <v>0</v>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199735232</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>1212499809</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>soonglobal</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>ビタ kダーククリアアイクリーム15ml リフィル</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F232" t="n">
+        <v>3724</v>
+      </c>
+      <c r="G232" t="n">
+        <v>0</v>
+      </c>
+      <c r="H232" t="b">
+        <v>0</v>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212499809</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>1206006286</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>ALLisWELL</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>ローズオブセッション ティント 24種（グロウ/マット）</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F233" t="n">
+        <v>1831</v>
+      </c>
+      <c r="G233" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" t="b">
+        <v>0</v>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206006286</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>1197650165</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>ALLisWELL</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>EFGセサル軟膏 5g / EGFクリーム (保湿ケア / 敏感肌サポート)</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>大熊製薬</t>
+        </is>
+      </c>
+      <c r="F234" t="n">
+        <v>2548</v>
+      </c>
+      <c r="G234" t="n">
+        <v>3</v>
+      </c>
+      <c r="H234" t="b">
+        <v>0</v>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197650165</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>1196294541</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>MALL-K</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>[正規品][ピジケア] ブランネイチャー アクネ クレンジングフォーム 企画 150ml（+50ml）</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>ブランナチュレ</t>
+        </is>
+      </c>
+      <c r="F235" t="n">
+        <v>4075</v>
+      </c>
+      <c r="G235" t="n">
+        <v>0</v>
+      </c>
+      <c r="H235" t="b">
+        <v>0</v>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196294541</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>1169175843</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>leewoostore</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>メイジング グレイス バレエローズ EDT 60ml</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Bella Philosophy</t>
+        </is>
+      </c>
+      <c r="F236" t="n">
+        <v>12947</v>
+      </c>
+      <c r="G236" t="n">
+        <v>0</v>
+      </c>
+      <c r="H236" t="b">
+        <v>0</v>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169175843</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>1211844368</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>leewoostore</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>ティーツリー シカ クーリング サンスティック リフィル企画 (20g+20g)</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F237" t="n">
+        <v>3429</v>
+      </c>
+      <c r="G237" t="n">
+        <v>0</v>
+      </c>
+      <c r="H237" t="b">
+        <v>0</v>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211844368</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>1210078286</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>leewoostore</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>[目元ケア] カフェインソリューション 5% + EGCG 30ml</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F238" t="n">
+        <v>2745</v>
+      </c>
+      <c r="G238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H238" t="b">
+        <v>0</v>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210078286</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>1210837026</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>leewoostore</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>セラムフィット UVプロテクター 01 クリア 50ml（SPF50+/PA++++)</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>ByUR</t>
+        </is>
+      </c>
+      <c r="F239" t="n">
+        <v>3211</v>
+      </c>
+      <c r="G239" t="n">
+        <v>0</v>
+      </c>
+      <c r="H239" t="b">
+        <v>0</v>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210837026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J221"/>
+  <autoFilter ref="A1:J239"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 63, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$239</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$255</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J239"/>
+  <dimension ref="A1:J255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10254,8 +10254,664 @@
         </is>
       </c>
     </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>1203335944</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>ボディローション ホワイトマスク520ml /韓国コスメ 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>ブーケガルニ</t>
+        </is>
+      </c>
+      <c r="F240" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G240" t="n">
+        <v>0</v>
+      </c>
+      <c r="H240" t="b">
+        <v>0</v>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203335944</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>1196699361</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>蓮花PDRNヒアルロン光彩セラム 30ml 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>ハンスキン</t>
+        </is>
+      </c>
+      <c r="F241" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G241" t="n">
+        <v>0</v>
+      </c>
+      <c r="H241" t="b">
+        <v>0</v>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196699361</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>1193167209</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>パンテノール クリーム 100ml 韓国スキンケア 韓国 コスメ #水分#保湿 毛穴ケア</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F242" t="n">
+        <v>4504</v>
+      </c>
+      <c r="G242" t="n">
+        <v>1</v>
+      </c>
+      <c r="H242" t="b">
+        <v>0</v>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193167209</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>1145411649</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>0liveshop</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>[保湿密封/しっかり水分パック] ナリシング トリートメント マスク 5枚/保湿マスク/乾燥対策/韓国コスメ/保湿トリートメントマスク/美肌マスク/敏感肌用マスク/シートマスク/トリートメントマスク</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F243" t="n">
+        <v>3010</v>
+      </c>
+      <c r="G243" t="n">
+        <v>0</v>
+      </c>
+      <c r="H243" t="b">
+        <v>0</v>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145411649</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>1146818611</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>thesugar</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>ペプチドショットアンプル 100ml x 2ea [大容量] / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F244" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G244" t="n">
+        <v>3</v>
+      </c>
+      <c r="H244" t="b">
+        <v>0</v>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146818611</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>1199411031</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Seoullys</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>[2+2] 白樺 水分 日焼け止めスプレー, 100ml 4ea(SPF 50 + PA ++++)</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F245" t="n">
+        <v>6007</v>
+      </c>
+      <c r="G245" t="n">
+        <v>0</v>
+      </c>
+      <c r="H245" t="b">
+        <v>0</v>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199411031</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>1136125175</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Seoullys</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>テラクネ 365 ハイドロ アクティブ トナー 化粧水, 200ml</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F246" t="n">
+        <v>2967</v>
+      </c>
+      <c r="G246" t="n">
+        <v>5</v>
+      </c>
+      <c r="H246" t="b">
+        <v>0</v>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136125175</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>1149907926</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>sssemibeauty</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>ブラックシュガーパーフェクトファーストセラム 150ml</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F247" t="n">
+        <v>2299</v>
+      </c>
+      <c r="G247" t="n">
+        <v>0</v>
+      </c>
+      <c r="H247" t="b">
+        <v>0</v>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149907926</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>1172085888</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>sssemibeauty</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>フルフィットプロポリスライトアンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F248" t="n">
+        <v>2337</v>
+      </c>
+      <c r="G248" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" t="b">
+        <v>0</v>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172085888</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>1203960088</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>345リリーフクリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F249" t="n">
+        <v>2453</v>
+      </c>
+      <c r="G249" t="n">
+        <v>1</v>
+      </c>
+      <c r="H249" t="b">
+        <v>0</v>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203960088</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>1192047927</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%トーニングソリューション 240ml トーニング ソリューション</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F250" t="n">
+        <v>2216</v>
+      </c>
+      <c r="G250" t="n">
+        <v>2</v>
+      </c>
+      <c r="H250" t="b">
+        <v>0</v>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192047927</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>1194225739</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>misssk</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>ソリッドパフューム7g 香り : レモンビヌ&amp;nbsp;/ バニラパーク 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>SENNOK</t>
+        </is>
+      </c>
+      <c r="F251" t="n">
+        <v>5366</v>
+      </c>
+      <c r="G251" t="n">
+        <v>0</v>
+      </c>
+      <c r="H251" t="b">
+        <v>0</v>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194225739</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>1173671918</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>misssk</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>ジェントルスキンクレンザー 473ml 大容量 コスパ 低刺激 乾燥肌 洗顔 敏感肌 クレンジング 肌荒れ /韓国コスメ/韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>セタフィル</t>
+        </is>
+      </c>
+      <c r="F252" t="n">
+        <v>2198</v>
+      </c>
+      <c r="G252" t="n">
+        <v>1</v>
+      </c>
+      <c r="H252" t="b">
+        <v>0</v>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173671918</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>1167121017</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>リンゼイ 鎮静薬草モデリングパック (カップパック) 28g [66冠/1位]</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LINDSAY</t>
+        </is>
+      </c>
+      <c r="F253" t="n">
+        <v>2278</v>
+      </c>
+      <c r="G253" t="n">
+        <v>1</v>
+      </c>
+      <c r="H253" t="b">
+        <v>0</v>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167121017</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>1204303349</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>ラエル オーガニックコットンカバー 履くオーバーナイト M 2個入 x3個</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>ラエル</t>
+        </is>
+      </c>
+      <c r="F254" t="n">
+        <v>3059</v>
+      </c>
+      <c r="G254" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" t="b">
+        <v>0</v>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204303349</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>1202040262</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>ジョソンアビューティ ワンダーバス レモンシロップ パッククレンザー 200ml (+50ml)</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>WONDER BATH</t>
+        </is>
+      </c>
+      <c r="F255" t="n">
+        <v>4332</v>
+      </c>
+      <c r="G255" t="n">
+        <v>0</v>
+      </c>
+      <c r="H255" t="b">
+        <v>0</v>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202040262</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J239"/>
+  <autoFilter ref="A1:J255"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 66, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$255</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$271</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J255"/>
+  <dimension ref="A1:J271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10910,8 +10910,664 @@
         </is>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>1203205247</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>vanguardvista</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>[正規品] 人気 おすすめ 韓国 クリーム Rx 30ml+7ml セット スキンケア クリーム ギフト</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>ドミナス</t>
+        </is>
+      </c>
+      <c r="F256" t="n">
+        <v>5820</v>
+      </c>
+      <c r="G256" t="n">
+        <v>0</v>
+      </c>
+      <c r="H256" t="b">
+        <v>0</v>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203205247</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>1165615884</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>ゼロ毛穴パッド2.0 70枚1セット</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F257" t="n">
+        <v>3372</v>
+      </c>
+      <c r="G257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H257" t="b">
+        <v>0</v>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165615884</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>1207138612</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>ビーネイチャー バナナ ホワイト マスクパック 10枚入</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F258" t="n">
+        <v>2422</v>
+      </c>
+      <c r="G258" t="n">
+        <v>0</v>
+      </c>
+      <c r="H258" t="b">
+        <v>0</v>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207138612</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>1207138588</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>プランシナジー シルキー マスクパック 10枚入</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F259" t="n">
+        <v>3087</v>
+      </c>
+      <c r="G259" t="n">
+        <v>0</v>
+      </c>
+      <c r="H259" t="b">
+        <v>0</v>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207138588</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>1165228864</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>ザリアルノニエネルギーアンプル30ml 1個</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F260" t="n">
+        <v>3087</v>
+      </c>
+      <c r="G260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H260" t="b">
+        <v>0</v>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165228864</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>1212496315</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>KONNI</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>ビタミンクリーム E 30ml</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Dr.VITA</t>
+        </is>
+      </c>
+      <c r="F261" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G261" t="n">
+        <v>0</v>
+      </c>
+      <c r="H261" t="b">
+        <v>0</v>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212496315</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>1206908379</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>onme</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>(+マスクパック贈呈)MGFリターンクリーム 70ml 再生クリーム</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>cellmedics</t>
+        </is>
+      </c>
+      <c r="F262" t="n">
+        <v>8600</v>
+      </c>
+      <c r="G262" t="n">
+        <v>0</v>
+      </c>
+      <c r="H262" t="b">
+        <v>0</v>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206908379</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>1136826440</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>onme</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>特許技術BBTMとともに安全に使用できる プレミアムビーガン女性用 プレミアム ビーガン 育毛シャンプー 韓国シャンプー 400ml</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>AGAIN ME</t>
+        </is>
+      </c>
+      <c r="F263" t="n">
+        <v>5050</v>
+      </c>
+      <c r="G263" t="n">
+        <v>1</v>
+      </c>
+      <c r="H263" t="b">
+        <v>0</v>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136826440</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>1123317400</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>withgaia</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>[1+1]レッド センテラカ マスク 10枚</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F264" t="n">
+        <v>7390</v>
+      </c>
+      <c r="G264" t="n">
+        <v>1</v>
+      </c>
+      <c r="H264" t="b">
+        <v>0</v>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123317400</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>1133684811</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>withgaia</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>プレミアムブリリアントミスト, 90ml</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Kopher</t>
+        </is>
+      </c>
+      <c r="F265" t="n">
+        <v>5350</v>
+      </c>
+      <c r="G265" t="n">
+        <v>0</v>
+      </c>
+      <c r="H265" t="b">
+        <v>0</v>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133684811</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>1203144925</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>ohnewcompany</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>【企画】オールアバウト グロウ カバークリーム (35g) + 大王パフ 1枚付き SPF50+ PA++++ 韓国コスメ ベースメイク 24時間持続 崩れない</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>CHASIN’ RABBITS</t>
+        </is>
+      </c>
+      <c r="F266" t="n">
+        <v>1946</v>
+      </c>
+      <c r="G266" t="n">
+        <v>1</v>
+      </c>
+      <c r="H266" t="b">
+        <v>0</v>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203144925</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>1160418590</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>julynana</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>[2種セット]ブリングリーン ティーツリー シカスージングトナー 250ml + クリーム100ml</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F267" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G267" t="n">
+        <v>0</v>
+      </c>
+      <c r="H267" t="b">
+        <v>0</v>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160418590</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>1152030824</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>julynana</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>[人気2種セット]ホワイトトリュフファーストスプレーセラム 100ml +ウォータフルトーンアップサンクリーム50ml</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F268" t="n">
+        <v>5640</v>
+      </c>
+      <c r="G268" t="n">
+        <v>0</v>
+      </c>
+      <c r="H268" t="b">
+        <v>0</v>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152030824</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>1134145901</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>allkbeauty</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>ダイブイン トナー 500ml+コットン60枚</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F269" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G269" t="n">
+        <v>0</v>
+      </c>
+      <c r="H269" t="b">
+        <v>0</v>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134145901</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>1134146014</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>allkbeauty</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>【新作追加/全5種】パフューム ヘアオイル 80ml+10ml/Angel muguet/La pitta/Hinoki/Osmanthus/Our leaf/perfumed hair oil</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>La'dor</t>
+        </is>
+      </c>
+      <c r="F270" t="n">
+        <v>4090</v>
+      </c>
+      <c r="G270" t="n">
+        <v>0</v>
+      </c>
+      <c r="H270" t="b">
+        <v>0</v>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134146014</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>1125176818</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>jandb</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>[PDRN4STEPセット]ピンクシカ スージングトナー+ピンクペプチド アンプル+PDRN ピンク ヒアルロニック 水分クリーム+ピンクエクソソームショット2000 or 7500</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F271" t="n">
+        <v>8990</v>
+      </c>
+      <c r="G271" t="n">
+        <v>1</v>
+      </c>
+      <c r="H271" t="b">
+        <v>0</v>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125176818</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J255"/>
+  <autoFilter ref="A1:J271"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 69, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$271</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$287</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J271"/>
+  <dimension ref="A1:J287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11566,8 +11566,664 @@
         </is>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>1161204302</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>kinakomall</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>[正規品]ドリクロ 20ml/脇汗デオドラント/デオドラント/脇汗/制汗剤/脇汗 韓国</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Driclor</t>
+        </is>
+      </c>
+      <c r="F272" t="n">
+        <v>1718</v>
+      </c>
+      <c r="G272" t="n">
+        <v>1</v>
+      </c>
+      <c r="H272" t="b">
+        <v>0</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161204302</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>1202451334</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>njhmall</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>ルフリージア オードパルファム 10ml</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>SISAO</t>
+        </is>
+      </c>
+      <c r="F273" t="n">
+        <v>4941</v>
+      </c>
+      <c r="G273" t="n">
+        <v>0</v>
+      </c>
+      <c r="H273" t="b">
+        <v>0</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202451334</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>1205580942</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>3番 ボドルボドル毛穴結セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F274" t="n">
+        <v>2561</v>
+      </c>
+      <c r="G274" t="n">
+        <v>0</v>
+      </c>
+      <c r="H274" t="b">
+        <v>0</v>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205580942</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>1203332451</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>ズーム バイ メイクアップ フィクサー 50ml 1+1</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>ZOOM BY JUNG SAEM MOOL</t>
+        </is>
+      </c>
+      <c r="F275" t="n">
+        <v>1876</v>
+      </c>
+      <c r="G275" t="n">
+        <v>0</v>
+      </c>
+      <c r="H275" t="b">
+        <v>0</v>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203332451</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>1205081404</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>[CU ビタミンU] アンプルトナー 130ml 1+1（皮膚科から始まったメディカルスキンケア）</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>CUSKIN</t>
+        </is>
+      </c>
+      <c r="F276" t="n">
+        <v>11119</v>
+      </c>
+      <c r="G276" t="n">
+        <v>0</v>
+      </c>
+      <c r="H276" t="b">
+        <v>0</v>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205081404</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>1208146662</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>アクネプロジェル30ml ニキビ肌の緩和機能性鎮静効果</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F277" t="n">
+        <v>4168</v>
+      </c>
+      <c r="G277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H277" t="b">
+        <v>0</v>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208146662</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>1211372508</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>[NEW]c-PDRNブースターショットジェルマスク 5枚 1個</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F278" t="n">
+        <v>4314</v>
+      </c>
+      <c r="G278" t="n">
+        <v>1</v>
+      </c>
+      <c r="H278" t="b">
+        <v>0</v>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211372508</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>1146074335</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>korkorhub</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>タヨースペシャルキッズバス友達セット6ラッチャキャリーティーチおもちゃミニカー車</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>tayo</t>
+        </is>
+      </c>
+      <c r="F279" t="n">
+        <v>2740</v>
+      </c>
+      <c r="G279" t="n">
+        <v>0</v>
+      </c>
+      <c r="H279" t="b">
+        <v>0</v>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146074335</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>1145379912</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>korkorhub</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>ダニエルトルースオイルパルファムナイトシェル10ml</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>DANIELS TRUTH</t>
+        </is>
+      </c>
+      <c r="F280" t="n">
+        <v>11800</v>
+      </c>
+      <c r="G280" t="n">
+        <v>0</v>
+      </c>
+      <c r="H280" t="b">
+        <v>0</v>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145379912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>1144242518</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>korkorhub</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>ブランディバレリーフティーツリーケアパッド 本品70+リフィル 70+70</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>blanc diva</t>
+        </is>
+      </c>
+      <c r="F281" t="n">
+        <v>8200</v>
+      </c>
+      <c r="G281" t="n">
+        <v>0</v>
+      </c>
+      <c r="H281" t="b">
+        <v>0</v>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1144242518</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>1189376677</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>velaskin</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>[NEW]シェイキング シナジー ミスト 50ml / 保湿ミスト / ツヤミスト / メイクキープ / うるおいケア / ミスト化粧水</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F282" t="n">
+        <v>3637</v>
+      </c>
+      <c r="G282" t="n">
+        <v>0</v>
+      </c>
+      <c r="H282" t="b">
+        <v>0</v>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189376677</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>1207185783</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>hadaluv</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>アロエエッセンスマスクパック1個入り50個</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>NatureBy</t>
+        </is>
+      </c>
+      <c r="F283" t="n">
+        <v>3525</v>
+      </c>
+      <c r="G283" t="n">
+        <v>0</v>
+      </c>
+      <c r="H283" t="b">
+        <v>0</v>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207185783</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>1207185764</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>hadaluv</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>ラグジュアリー24kゴールドアンプル100ml 1個</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F284" t="n">
+        <v>2585</v>
+      </c>
+      <c r="G284" t="n">
+        <v>0</v>
+      </c>
+      <c r="H284" t="b">
+        <v>0</v>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207185764</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>1207185727</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>hadaluv</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>アロエ97％スーディングジェル300ml 2個入りポムポムプリン</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F285" t="n">
+        <v>4747</v>
+      </c>
+      <c r="G285" t="n">
+        <v>0</v>
+      </c>
+      <c r="H285" t="b">
+        <v>0</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207185727</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>1207183624</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>hadaluv</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>ブライトニングヒアルロンフィリングジェル170ml 2個</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F286" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G286" t="n">
+        <v>0</v>
+      </c>
+      <c r="H286" t="b">
+        <v>0</v>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207183624</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>1213161313</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>pinnacosme</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>アンリミテッドメイクアップフィックスミストマット, 100ml</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>シュウウエムラ</t>
+        </is>
+      </c>
+      <c r="F287" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G287" t="n">
+        <v>0</v>
+      </c>
+      <c r="H287" t="b">
+        <v>0</v>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213161313</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J271"/>
+  <autoFilter ref="A1:J287"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 72, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$287</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$303</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J287"/>
+  <dimension ref="A1:J303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12222,8 +12222,664 @@
         </is>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>1207330609</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>joohoh2</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>[メンズ オールインワン 限定企画3種セット] アクアパワー オールインワン 200ml セット ＋クレンザー40ml／オールインワン20ml 付き</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>ビオテルム</t>
+        </is>
+      </c>
+      <c r="F288" t="n">
+        <v>5292</v>
+      </c>
+      <c r="G288" t="n">
+        <v>0</v>
+      </c>
+      <c r="H288" t="b">
+        <v>0</v>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207330609</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>1189316227</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>theories</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>[PDRN 限定セット] ダーマヒーラーポアタイトニングアンプル30ml + トナーパッド2枚 X 6ea</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F289" t="n">
+        <v>5157</v>
+      </c>
+      <c r="G289" t="n">
+        <v>0</v>
+      </c>
+      <c r="H289" t="b">
+        <v>0</v>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189316227</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>1178929059</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>theories</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>[男女共用ヘアラインクッション] デイリースリムクイックヘアーラインクッション/2タイプ から選択</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F290" t="n">
+        <v>2403</v>
+      </c>
+      <c r="G290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H290" t="b">
+        <v>0</v>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178929059</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>1152467548</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>theories</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>[40代女性 シワケア必須アイテム] リンクル リペア ほうれい線 パッチ 36個入り</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>MARSHIQUE</t>
+        </is>
+      </c>
+      <c r="F291" t="n">
+        <v>1651</v>
+      </c>
+      <c r="G291" t="n">
+        <v>0</v>
+      </c>
+      <c r="H291" t="b">
+        <v>0</v>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152467548</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>1180574367</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>fromAnswer</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>[10Sマイクロバブルパック 4種] エア** バブルCDS マスク パック 80ml, 4種の中から選択 (ハリ/ブライトニング/鎮静/水分) 150 回分</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Gear By Gash</t>
+        </is>
+      </c>
+      <c r="F292" t="n">
+        <v>4014</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0</v>
+      </c>
+      <c r="H292" t="b">
+        <v>0</v>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180574367</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>1189270361</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>【Wid】 フォリゲン トニック 120ml 2個セット・頭皮ケア・ヘアトニック・抜け毛予防・頭皮栄養・スカルプケア</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F293" t="n">
+        <v>5287</v>
+      </c>
+      <c r="G293" t="n">
+        <v>0</v>
+      </c>
+      <c r="H293" t="b">
+        <v>0</v>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189270361</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>1188452071</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>【Wid】 アスコルビルテトラィソパルミテート ソリューション 20% イン ビタミンF / 30ml / 1個 / ビタミンC美容液 / オイル美容液 / 透明感 / ハリケア</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F294" t="n">
+        <v>5841</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0</v>
+      </c>
+      <c r="H294" t="b">
+        <v>0</v>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452071</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>1188452072</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>【Wid】 グリコール酸 7% エクスフォリエイティング トナー / 240ml / 2個セット / ふき取り化粧水 / 角質ケア / 肌キメ整え / ツヤ肌</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>6385</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0</v>
+      </c>
+      <c r="H295" t="b">
+        <v>0</v>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452072</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>1179809144</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>[角質ケア] マンデル酸 10％ + HA 30ml 毛穴ケア つるつる美肌 セラム</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>2485</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="b">
+        <v>0</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179809144</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>1174312286</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>【1+1】【韓国コスメ】【正規品扱い店】[病院専用] ラポラピルナトックス 50ml - シミ改善＆肌トーンアップの機能性クリーム！</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Dermagen</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>7128</v>
+      </c>
+      <c r="G297" t="n">
+        <v>0</v>
+      </c>
+      <c r="H297" t="b">
+        <v>0</v>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174312286</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>1146499682</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】タイムエナジーリセッティングエマルジョン 120ml - 時間を超える美肌の秘訣！</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F298" t="n">
+        <v>4781</v>
+      </c>
+      <c r="G298" t="n">
+        <v>0</v>
+      </c>
+      <c r="H298" t="b">
+        <v>0</v>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146499682</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>1146499598</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】[5番企画セット] 白玉リンガーグルタチオンCトナー200ML ＋ 白玉グルタチオンC美容液30ML - 輝く美肌へ導く！</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>7013</v>
+      </c>
+      <c r="G299" t="n">
+        <v>0</v>
+      </c>
+      <c r="H299" t="b">
+        <v>0</v>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146499598</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>1145594895</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>sinature22</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>【正規品扱い店】【1+1】【本品+レフィル】ダイブイン低分子ヒアルロン酸セラム, 50mL*2</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>4879</v>
+      </c>
+      <c r="G300" t="n">
+        <v>0</v>
+      </c>
+      <c r="H300" t="b">
+        <v>0</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145594895</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>1145594718</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>sinature22</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】シルクペプチドインテンシブリフティングアンプル35ML</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>2407</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0</v>
+      </c>
+      <c r="H301" t="b">
+        <v>0</v>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145594718</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>1145562017</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>ecoon5629</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】インテカ スージングクリーム 80ml（＋クリーム31ml）</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>メイクプレム</t>
+        </is>
+      </c>
+      <c r="F302" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0</v>
+      </c>
+      <c r="H302" t="b">
+        <v>0</v>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145562017</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>1145561724</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>ecoon5629</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】シカ80ヒアルロン酸トナー260mL - 敏感肌を優しく守る潤いの秘訣！</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>frankly</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>2897</v>
+      </c>
+      <c r="G303" t="n">
+        <v>2</v>
+      </c>
+      <c r="H303" t="b">
+        <v>0</v>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145561724</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J287"/>
+  <autoFilter ref="A1:J303"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 75, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$319</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J303"/>
+  <dimension ref="A1:J319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12878,8 +12878,664 @@
         </is>
       </c>
     </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>1210528997</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>【1+1セット】クリーンティーツリーリポソーム カーミングマスク 5枚入×2個 ヒアルロン酸 パンテノール 水分 鎮静 保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F304" t="n">
+        <v>3069</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0</v>
+      </c>
+      <c r="H304" t="b">
+        <v>0</v>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210528997</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>1210272622</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>【1+1セット】ウォータフルエッセンスサンクリーム SPF50+ PA++++ 50ml×2個 保湿 UVケア エッセンス 日焼け止め 化粧下地 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>6442</v>
+      </c>
+      <c r="G305" t="n">
+        <v>0</v>
+      </c>
+      <c r="H305" t="b">
+        <v>0</v>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210272622</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>1206508858</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>【1+1セット】ソフトリセット グリーンクレンジングバーム 100ml 2個 メイク落とし 保湿洗顔 角質ケア 毛穴汚れケア 韓国コスメ しっとりディープクレンジング</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>ヒュッゲ</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>6279</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+      <c r="H306" t="b">
+        <v>0</v>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206508858</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>1206240655</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>ウォーターtoアンプルトリートメント 200ml 1個 毛髪保湿 ツヤ髪ケア しっとりヘアケア ホームケア 韓国コスメ 上品な香り デイリーケア</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>6459</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0</v>
+      </c>
+      <c r="H307" t="b">
+        <v>0</v>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206240655</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>1209385608</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>woozshop</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>プシュケシロップジェル8種単品 (10ml) / デイリーネイル /ヌードトーンネイル/シロップネイル/シロップジェル/ウェディングネイル/韓国ネイル</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>FROM THE NAIL</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" t="b">
+        <v>0</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209385608</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>1205917792</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>woozshop</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>ローズコア磁石 6種 10g 1個 / マグネットネイル/ サロンネイル/ ローズネイル</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>FROM THE NAIL</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="b">
+        <v>0</v>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205917792</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>1212657160</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>kacos</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>レッドトマト ジェリーリップマスク / グリーントマト スムージーリップスクラブ 12g</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>FULLY</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H310" t="b">
+        <v>0</v>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212657160</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>1183884384</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>haruharukorea</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>【NEW/新商品 PDRN】PDRNピンクゼリーセラムミスト 100ml /韓国コスメ ハリ 弾力 保湿ミスト 美容液 霧噴射 ツヤ 毛穴ケア 弾力ケア メイクキープ コラーゲン グルタチオン</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>3490</v>
+      </c>
+      <c r="G311" t="n">
+        <v>1</v>
+      </c>
+      <c r="H311" t="b">
+        <v>0</v>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183884384</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>1183042681</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>haruharukorea</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>【NEW/新商品 PDRN】ヒアルロン酸ハイドレイティングミスト 100ml /韓国コスメ ハリ 弾力 保湿ミスト フェイスミスト 霧噴射 ツヤ 角質ケア 毛穴ケア 弾力ケア メイクキープ</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>3790</v>
+      </c>
+      <c r="G312" t="n">
+        <v>2</v>
+      </c>
+      <c r="H312" t="b">
+        <v>0</v>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183042681</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>1208052392</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>haruharukorea</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>【Q10人気 ゼロ毛穴美容液】ゼロ毛穴エクソソームショット2000 30ml/毛穴美容液 ナイアシンアミド美容液 針美容液 毛穴の黒ずみ 皮脂 角質トラブルケア パンテノール 脂性肌</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" t="b">
+        <v>0</v>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208052392</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>1165596406</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>haruharukorea</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>【Q10超おすすめ】ホワイトトリュフバイタルスプレーセラム, 100ml/水分/鎮静/保湿/栄養/弾力/腰/光彩/ツヤ/霧噴射/ツヤ肌/メイクキープ /ミスト セラム/保湿美容液/美容液/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>3950</v>
+      </c>
+      <c r="G314" t="n">
+        <v>1</v>
+      </c>
+      <c r="H314" t="b">
+        <v>0</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165596406</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>1159803084</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>haruharukorea</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>【正規品】 デュアル エフェクト アンプル 30mL , 2本セット/PDRN ( c-PDRN )/美容液/ゴールド スキンケア /みずみずしい美容液/水ツヤ肌//保湿アンプル/マルチケア集中美容液</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>12799</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0</v>
+      </c>
+      <c r="H315" t="b">
+        <v>0</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159803084</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>1193925287</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>sara_korea</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>【韓国 化粧品】[1+1] 脱毛緩和 フォリゲンシャンプー, 500ml 2個 /(脱毛症状ケア/ボリューム強化)</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>4633</v>
+      </c>
+      <c r="G316" t="n">
+        <v>1</v>
+      </c>
+      <c r="H316" t="b">
+        <v>0</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193925287</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>1190719334</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>sara_korea</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>【韓国 化粧品】デイリーモイスチャーボディローション, 400ml 1個 /韓国で人気の保湿クリーム</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>ダーマビー</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>1937</v>
+      </c>
+      <c r="G317" t="n">
+        <v>1</v>
+      </c>
+      <c r="H317" t="b">
+        <v>0</v>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190719334</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>1206710414</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>k-wonderland</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>超高含有ヒアルロニックインテンストナー 100時間保湿持続力300g</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>3148</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0</v>
+      </c>
+      <c r="H318" t="b">
+        <v>0</v>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206710414</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>1209385392</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>k-wonderland</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>アドール パフューム ヘアオイル 80ml 5種類から選べる</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>アドル</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>3456</v>
+      </c>
+      <c r="G319" t="n">
+        <v>1</v>
+      </c>
+      <c r="H319" t="b">
+        <v>0</v>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209385392</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J303"/>
+  <autoFilter ref="A1:J319"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 78, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$319</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$328</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J319"/>
+  <dimension ref="A1:J328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13534,8 +13534,377 @@
         </is>
       </c>
     </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>1187728361</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>cosmeticmall</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>TXシミ取りクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F320" t="n">
+        <v>2425</v>
+      </c>
+      <c r="G320" t="n">
+        <v>3</v>
+      </c>
+      <c r="H320" t="b">
+        <v>0</v>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187728361</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>1194254316</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>kanikemen</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>【正規品】 サロン10 シャンプー + トリートメント セット （シカプロテインシャンプー 480ml + シカプロテイントリートメント 215ml）</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G321" t="n">
+        <v>0</v>
+      </c>
+      <c r="H321" t="b">
+        <v>0</v>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194254316</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>1207580983</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>kanikemen</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>【正規品】 1+1 計2個 グルタチオンセブンダークスポットセラム 30ml 2個</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G322" t="n">
+        <v>0</v>
+      </c>
+      <c r="H322" t="b">
+        <v>0</v>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207580983</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>1211973120</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>eloisestore</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>【ポケモンエディション】カラーグラム タンフル リップセラム 9色 キーリング付属</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>カラーグラム</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>1698</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0</v>
+      </c>
+      <c r="H323" t="b">
+        <v>0</v>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211973120</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>1080883557</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>eloisestore</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>ドクターペプチドボリュームリフティングプロエッセンス100ml 2個</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>DR.PEPTI</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>13200</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0</v>
+      </c>
+      <c r="H324" t="b">
+        <v>0</v>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080883557</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>1203766483</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>ウォータープルーフ サーフィン サンスティック 20g</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>3201</v>
+      </c>
+      <c r="G325" t="n">
+        <v>0</v>
+      </c>
+      <c r="H325" t="b">
+        <v>0</v>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203766483</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>1096782550</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>アクア ヒアルロニック エッセンス 大容量, 250ml</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>3888</v>
+      </c>
+      <c r="G326" t="n">
+        <v>0</v>
+      </c>
+      <c r="H326" t="b">
+        <v>0</v>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096782550</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>1168004689</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>ruimay</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>パフュームシャンプー+リンスセッ[スイートパラウォーリー/フレッシュラッシュ/バイオレット/グリーンリリー/ホワイトデイジー]ツヤ 栄養 保湿 水分 香水 シャンプー 柔らかな髪で韓国の人気シャンプー</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>2744</v>
+      </c>
+      <c r="G327" t="n">
+        <v>0</v>
+      </c>
+      <c r="H327" t="b">
+        <v>0</v>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168004689</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>1132024666</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>happybear</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>[MARTINA GEBHARDT] アボカド アイクリーム 15ml</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>マルティナ</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G328" t="n">
+        <v>1</v>
+      </c>
+      <c r="H328" t="b">
+        <v>0</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132024666</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J319"/>
+  <autoFilter ref="A1:J328"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 81, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$328</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$342</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J328"/>
+  <dimension ref="A1:J342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13903,8 +13903,582 @@
         </is>
       </c>
     </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>1128158961</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Glowme</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>[公式]韓国で売れてます / しみ取りクリーム / しみ / そばかす / くすみ / トーンアップクリーム / ピュアビタミンC 1% ナイアシンアミド5% 配合 - ブライトニングクリーム</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>HWASA</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>1750</v>
+      </c>
+      <c r="G329" t="n">
+        <v>2</v>
+      </c>
+      <c r="H329" t="b">
+        <v>0</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1128158961</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>1194573796</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュクリアスージングクリーム, 70ml, 2個</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0</v>
+      </c>
+      <c r="H330" t="b">
+        <v>0</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194573796</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>1213387450</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Crystal_K</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>THEVITAレチナールショットタイトニングブースター, 15ml, 2個</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>3020</v>
+      </c>
+      <c r="G331" t="n">
+        <v>0</v>
+      </c>
+      <c r="H331" t="b">
+        <v>0</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213387450</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>1168692108</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>【正規品】松の木 鎮静 シカ クレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G332" t="n">
+        <v>0</v>
+      </c>
+      <c r="H332" t="b">
+        <v>0</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168692108</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>1164469069</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>【正規品】グリーンシカ コラーゲン クリアフォーム 2.0 300ml</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="b">
+        <v>0</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164469069</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>1163729695</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>【正規品】ディープポア クレンジング ソーダフォーム 150ml</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
+      <c r="H334" t="b">
+        <v>0</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163729695</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>1205554253</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>【正規品】トラネキサム酸スキンブースタークリーム 100ml</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>メディテラピー</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0</v>
+      </c>
+      <c r="H335" t="b">
+        <v>0</v>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205554253</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>1193459511</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>【正規品】レチノコラーゲン低分子300ネックカッサクリーム 50ml (2個)</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>CKD_GUARANTEED</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>6490</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0</v>
+      </c>
+      <c r="H336" t="b">
+        <v>0</v>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193459511</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>1159224305</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>jaenypick</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>シカフルアンプル30ml 1個</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>1894</v>
+      </c>
+      <c r="G337" t="n">
+        <v>1</v>
+      </c>
+      <c r="H337" t="b">
+        <v>0</v>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159224305</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>1149395148</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>jaenypick</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド 20% セラム80ml1個</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>2473</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0</v>
+      </c>
+      <c r="H338" t="b">
+        <v>0</v>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149395148</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>1200324318</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>jaenypick</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>ヒアルロン酸2% + B5 セラム 30ml 1個</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>2671</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0</v>
+      </c>
+      <c r="H339" t="b">
+        <v>0</v>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200324318</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>1197354746</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>jaenypick</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>345 リリーフクリームミスト1個 100ml</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F340" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0</v>
+      </c>
+      <c r="H340" t="b">
+        <v>0</v>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197354746</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>1087617512</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>QueenMall</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>パフューム スプレー ボディローション 250ml 5種</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>hedn</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>4320</v>
+      </c>
+      <c r="G341" t="n">
+        <v>1</v>
+      </c>
+      <c r="H341" t="b">
+        <v>0</v>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1087617512</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>1170080586</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>QueenMall</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>PDRN ピンク ジェル ツーフォーム クレンザー 200ml 企画(+クレンジングブラシ 贈呈)</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>2972</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
+      <c r="H342" t="b">
+        <v>0</v>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170080586</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J328"/>
+  <autoFilter ref="A1:J342"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 84, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$342</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$355</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J342"/>
+  <dimension ref="A1:J355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14477,8 +14477,541 @@
         </is>
       </c>
     </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>1199098148</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>kiri</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>[モンチッチコラボ] ベージュトーンアップ365ヴィーガンサンクリーム 40ml SPF50 トーンアップUV ノーファンデ 化粧下地 韓国日焼け止め</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>アミューズ</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>3470</v>
+      </c>
+      <c r="G343" t="n">
+        <v>1</v>
+      </c>
+      <c r="H343" t="b">
+        <v>0</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199098148</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>1211134600</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>seimyongkorea</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>【NEW】 シェイキングミスト</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>2222</v>
+      </c>
+      <c r="G344" t="n">
+        <v>2</v>
+      </c>
+      <c r="H344" t="b">
+        <v>0</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211134600</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>1109779971</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>[V T] リードルショット 2ステップ マスク 5枚セット (50/100/300) 針美容 毛穴 導入 フェイスパック 集中ケア スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>2739</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0</v>
+      </c>
+      <c r="H345" t="b">
+        <v>0</v>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109779971</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>1192596376</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>[メガ割] manyo factory 魔女工場 ガラクナイアシン エッセンス クリーム 50ml ガラクトミセス 保湿 弾力 ハリ ツヤ 潤い 浸透 スキンケア 基礎化粧品 韓国コスメ 人気 公式</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>4726</v>
+      </c>
+      <c r="G346" t="n">
+        <v>0</v>
+      </c>
+      <c r="H346" t="b">
+        <v>0</v>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192596376</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>1193869990</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>K--beautyshop</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>[1+1特典] S*NATURE エ*スネイチャー アクア スクワラン 水分クリーム 2個セット 120ml 保湿 ツヤ肌 卵肌 韓国 スキンケア オリーブヤング プレゼント 敏感肌 乾燥肌</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>エスネイチャー</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>3930</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0</v>
+      </c>
+      <c r="H347" t="b">
+        <v>0</v>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193869990</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>1183178551</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Starlit</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>TN トラネキサミン5%＋ナイアシンアミド5% ブライトニング セラム60ml</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>コスデバハ</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>3880</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0</v>
+      </c>
+      <c r="H348" t="b">
+        <v>0</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183178551</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>1188405527</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Starlit</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>ゆずグレープフルーツ ビーガン パッククレンザー 80g+毛穴ブラシ [毛穴ケア+洗顔+すっきり]</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>ホイップド</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G349" t="n">
+        <v>0</v>
+      </c>
+      <c r="H349" t="b">
+        <v>0</v>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188405527</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>1188406613</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Starlit</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>セラミド アト ローション 600ml [保湿+バリア+敏感肌]</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>3040</v>
+      </c>
+      <c r="G350" t="n">
+        <v>1</v>
+      </c>
+      <c r="H350" t="b">
+        <v>0</v>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188406613</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>1102457193</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>JJDD</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>ブランマジックティーツリーオイル 20ml 5倍高濃縮ティーツリー成分 /ニキビ超急速ケア/赤ニキビ,白ニキビ,大人ニキビ,思春期ニキビ,ニキビ跡</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>ブランネイチャー</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>2350</v>
+      </c>
+      <c r="G351" t="n">
+        <v>1</v>
+      </c>
+      <c r="H351" t="b">
+        <v>0</v>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102457193</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>1188402180</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>EGF ポストレーザー セラムミスト 120ml [再生+鎮静+ミスト]</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>イージーデュー</t>
+        </is>
+      </c>
+      <c r="F352" t="n">
+        <v>5130</v>
+      </c>
+      <c r="G352" t="n">
+        <v>1</v>
+      </c>
+      <c r="H352" t="b">
+        <v>0</v>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188402180</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>1188402173</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>アロエ スージングジェルミスト 155ml×3 [鎮静+保湿+時短]</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F353" t="n">
+        <v>2940</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0</v>
+      </c>
+      <c r="H353" t="b">
+        <v>0</v>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188402173</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>1188402116</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>ダーマアンサー PDRN アンプル 30ml+60ml リフィル [弾力+保湿+セット]</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>CNP Laboratory</t>
+        </is>
+      </c>
+      <c r="F354" t="n">
+        <v>5410</v>
+      </c>
+      <c r="G354" t="n">
+        <v>0</v>
+      </c>
+      <c r="H354" t="b">
+        <v>0</v>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188402116</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>1210683594</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>82lounge</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>メディAHAクリーム 25ml :: AHAクリーム / クリーム 角質除去 / クリーム スポットケア / クリーム ニキビ</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F355" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G355" t="n">
+        <v>0</v>
+      </c>
+      <c r="H355" t="b">
+        <v>0</v>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210683594</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J342"/>
+  <autoFilter ref="A1:J355"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 87, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$355</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$371</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J355"/>
+  <dimension ref="A1:J371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15010,8 +15010,664 @@
         </is>
       </c>
     </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>1169201226</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>[1+1]ジェントルブラック フレッシュ クレンジングオイル 150ml+150ml</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>dear,Klairs</t>
+        </is>
+      </c>
+      <c r="F356" t="n">
+        <v>4584</v>
+      </c>
+      <c r="G356" t="n">
+        <v>0</v>
+      </c>
+      <c r="H356" t="b">
+        <v>0</v>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169201226</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>1110101930</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>フォリゲンシャンプー 500ml</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>2847</v>
+      </c>
+      <c r="G357" t="n">
+        <v>0</v>
+      </c>
+      <c r="H357" t="b">
+        <v>0</v>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110101930</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>1092755563</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>JSKSHOPPING</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>ベイキング パウダー サクサク 毛穴 スクラブ 200gx2個</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>エチュード</t>
+        </is>
+      </c>
+      <c r="F358" t="n">
+        <v>3148</v>
+      </c>
+      <c r="G358" t="n">
+        <v>5</v>
+      </c>
+      <c r="H358" t="b">
+        <v>0</v>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1092755563</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>1203684966</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>elom トラブルスケーリングパッチマスク 3枚 /トラブルケア</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>EIoM</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0</v>
+      </c>
+      <c r="H359" t="b">
+        <v>0</v>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203684966</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>1179656795</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>こすアールエックス ワンステップパッド/おじさんパッド/ピンプルパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F360" t="n">
+        <v>3490</v>
+      </c>
+      <c r="G360" t="n">
+        <v>0</v>
+      </c>
+      <c r="H360" t="b">
+        <v>0</v>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179656795</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>1190674241</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>KBeautyCenter</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>カロテンクラリファイングビタパッド, 60枚</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0</v>
+      </c>
+      <c r="H361" t="b">
+        <v>0</v>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190674241</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>1083089713</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>fresh-aka</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>ピュアフィットシカ 弱酸性クレンジングパッド 100枚入 * 1個</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G362" t="n">
+        <v>0</v>
+      </c>
+      <c r="H362" t="b">
+        <v>0</v>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083089713</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>1082221247</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>fresh-aka</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>ムード ペブル ネイル 29種</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>ロムアンド</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G363" t="n">
+        <v>0</v>
+      </c>
+      <c r="H363" t="b">
+        <v>0</v>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1082221247</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>1209886899</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>osondoson7</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>もちもちチョコ 餅パイ 大容量 40個入り 860g</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>チョンウ食品</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>3042</v>
+      </c>
+      <c r="G364" t="n">
+        <v>0</v>
+      </c>
+      <c r="H364" t="b">
+        <v>0</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209886899</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>1180517208</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>osondoson7</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュクリアヒアルシカスーディングセラム50ml1個</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0</v>
+      </c>
+      <c r="H365" t="b">
+        <v>0</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180517208</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>1208425109</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>osondoson7</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>シークレットライス麹ピーリングツーフォームクレンザー120g1個</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>3827</v>
+      </c>
+      <c r="G366" t="n">
+        <v>1</v>
+      </c>
+      <c r="H366" t="b">
+        <v>0</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208425109</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>1188886447</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>RANIBEAUTY</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>【サンプル5枚】イニスフリー グリーンティーシリーズ/ヒアルロン酸/スキン/ローション/クリーム/シードセラム/アミノ クレンジングフォーム/ウォーター/オイル/アイ＆フェイスボール</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0</v>
+      </c>
+      <c r="H367" t="b">
+        <v>0</v>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188886447</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>1205550323</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>dgrm</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>リジュラン ダーマ ヒーラー ポア タイトニング トナー パッド 220mL</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>3960</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0</v>
+      </c>
+      <c r="H368" t="b">
+        <v>0</v>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205550323</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>1177829431</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>dgrm</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>マイファーストセラム 50ml</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>De:maf</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>2430</v>
+      </c>
+      <c r="G369" t="n">
+        <v>0</v>
+      </c>
+      <c r="H369" t="b">
+        <v>0</v>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177829431</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>1180354766</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>[1+1/限定企画] スキンフード キャロット カロチン カミング ウォーターパッド 60枚 ダブル企画</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F370" t="n">
+        <v>6791</v>
+      </c>
+      <c r="G370" t="n">
+        <v>0</v>
+      </c>
+      <c r="H370" t="b">
+        <v>0</v>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180354766</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>1207273381</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>PDRN ピンク コラーゲン バーム セラム 95ml 炭酸 泡 美容液 水光肌 弾力 ほうれい線 乾燥肌 エイジングケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F371" t="n">
+        <v>5049</v>
+      </c>
+      <c r="G371" t="n">
+        <v>0</v>
+      </c>
+      <c r="H371" t="b">
+        <v>0</v>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207273381</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J355"/>
+  <autoFilter ref="A1:J371"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 90, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$371</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$380</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J371"/>
+  <dimension ref="A1:J380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15666,8 +15666,377 @@
         </is>
       </c>
     </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>1205150670</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>shoplikable</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>[1+1+ミニ6枚付き/大容量企画] ポアタイトニング トナーパッド 60枚 ダブル企画 毛穴ケア 韓国パッド 角質ケア 保湿パッド</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F372" t="n">
+        <v>4398</v>
+      </c>
+      <c r="G372" t="n">
+        <v>0</v>
+      </c>
+      <c r="H372" t="b">
+        <v>0</v>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205150670</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>1193784439</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>shoplikable</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>【大容量・本品＋詰め替え】 グローターン エクソソーム ブラシアンプル 100ml＋リフィル100ml 頭皮ケア スカルプ美容液 抜け毛・ハリコシケア</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F373" t="n">
+        <v>5661</v>
+      </c>
+      <c r="G373" t="n">
+        <v>0</v>
+      </c>
+      <c r="H373" t="b">
+        <v>0</v>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193784439</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>1207091863</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>リードルショット フォーメン オールインワン100 Mプラス 150ml＋30ml 企画セット メンズスキンケア 韓国コスメ 化粧水 乳液 美容液</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F374" t="n">
+        <v>3855</v>
+      </c>
+      <c r="G374" t="n">
+        <v>0</v>
+      </c>
+      <c r="H374" t="b">
+        <v>0</v>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091863</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>1174137858</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>ローズマリー &amp;amp; シーソルト &amp;amp; AHA シャンプー 500ml × 2本セット 韓国シャンプー スカルプケア 頭皮クレンジング ボリュームケア</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>オーガニスト</t>
+        </is>
+      </c>
+      <c r="F375" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G375" t="n">
+        <v>0</v>
+      </c>
+      <c r="H375" t="b">
+        <v>0</v>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174137858</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>1024539184</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>[1+1]ハニーアンドマカデミア ネイチャーシャンプー 500ml+プロテイントリートメント 500mlホワイトムスクの香り</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F376" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G376" t="n">
+        <v>1</v>
+      </c>
+      <c r="H376" t="b">
+        <v>0</v>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1024539184</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>1207091851</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>kyo_market</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>3番 ノーファンデ陶器肌トーンアップUVクリーム 50ml (SPF50+ PA++++) / トーンケアクリーム 保湿ベース 水分クリーム 化粧下地 ナチュラルトーンアップ</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G377" t="n">
+        <v>0</v>
+      </c>
+      <c r="H377" t="b">
+        <v>0</v>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091851</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>1112935346</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>【選べる2個セット】デビルズ パフュームファンタジーシャンプー &amp;amp; コンディショナー, 1L+1L</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G378" t="n">
+        <v>1</v>
+      </c>
+      <c r="H378" t="b">
+        <v>0</v>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1112935346</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>1084157476</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>【NEW COLOR】イージーブロウトーンチェンジャー (5回分) /ブリーチ / 眉毛脱色 /眉カラーケア</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>サムバイミー</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>4110</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0</v>
+      </c>
+      <c r="H379" t="b">
+        <v>0</v>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1084157476</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>1209812267</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>thebest_mall</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>SOSセラム, 50ml</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>3524</v>
+      </c>
+      <c r="G380" t="n">
+        <v>0</v>
+      </c>
+      <c r="H380" t="b">
+        <v>0</v>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209812267</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J371"/>
+  <autoFilter ref="A1:J380"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 93, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$380</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$398</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J380"/>
+  <dimension ref="A1:J398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16035,8 +16035,746 @@
         </is>
       </c>
     </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>1191781202</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>MEDIHEAL トナーパッド2.0 リフィル 70枚×2個セット 4タイプ選択可</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>1918</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0</v>
+      </c>
+      <c r="H381" t="b">
+        <v>0</v>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191781202</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>1204359324</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>【1+1 / SNS話題】ツヤ肌バブルエッセンストナー 95ml</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>curest</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>2131</v>
+      </c>
+      <c r="G382" t="n">
+        <v>0</v>
+      </c>
+      <c r="H382" t="b">
+        <v>0</v>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204359324</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>1160562706</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>pepeshop</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>アトバリア365クリームミスト 120ml</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G383" t="n">
+        <v>3</v>
+      </c>
+      <c r="H383" t="b">
+        <v>0</v>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160562706</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>1203402766</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>pepeshop</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>【5月新作/Qoo10先行発売】ザ・ブルーペプチド バクチオール 縦毛穴 セラム 50mL</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G384" t="n">
+        <v>1</v>
+      </c>
+      <c r="H384" t="b">
+        <v>0</v>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203402766</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>1199565099</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>pepeshop</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>デリケートゾーン 黒ずみ クリーム ナイアシンアミド 公式 アンダーアームクリーム 100g</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>BnD</t>
+        </is>
+      </c>
+      <c r="F385" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0</v>
+      </c>
+      <c r="H385" t="b">
+        <v>0</v>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199565099</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>1210391803</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>pepeshop</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>【新商品】 3番 キメブースター時短バブルパック, 90ml</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F386" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G386" t="n">
+        <v>0</v>
+      </c>
+      <c r="H386" t="b">
+        <v>0</v>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210391803</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>1171947071</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>【正規品】 デイリートナーパッド 80枚</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>NEEDLY</t>
+        </is>
+      </c>
+      <c r="F387" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G387" t="n">
+        <v>0</v>
+      </c>
+      <c r="H387" t="b">
+        <v>0</v>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171947071</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>1171946936</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>【正規品】 センテラクイックカーミングパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F388" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G388" t="n">
+        <v>3</v>
+      </c>
+      <c r="H388" t="b">
+        <v>0</v>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171946936</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>1197892266</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>【正規品】 グロウクリーミーボディスクラブ ヌバニラ 300ml</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F389" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G389" t="n">
+        <v>0</v>
+      </c>
+      <c r="H389" t="b">
+        <v>0</v>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197892266</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>1205623680</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Ohharu</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>[正規品]NEW アトバリア365 カプセルトナー 300ml,リニューアルアトバリア365 ハイドロスーディングクリーム 80ml/化粧水/クリーム/ニキビ/韓国コスメ 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F390" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0</v>
+      </c>
+      <c r="H390" t="b">
+        <v>0</v>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205623680</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>1197665370</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>オンリーフォーマンオールインワンエッセンス 200ml 2個 皮脂ケア テカリ防止</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F391" t="n">
+        <v>5683</v>
+      </c>
+      <c r="G391" t="n">
+        <v>0</v>
+      </c>
+      <c r="H391" t="b">
+        <v>0</v>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665370</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>1197665508</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュフォーマン鎮静オールインワン 200ml 3個 お得 ストック</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F392" t="n">
+        <v>12618</v>
+      </c>
+      <c r="G392" t="n">
+        <v>0</v>
+      </c>
+      <c r="H392" t="b">
+        <v>0</v>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665508</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>1197665474</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>メンズグッドルックスアイブローペンシル ナチュラルブラック 1個 目力 男子メイク</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F393" t="n">
+        <v>1921</v>
+      </c>
+      <c r="G393" t="n">
+        <v>0</v>
+      </c>
+      <c r="H393" t="b">
+        <v>0</v>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665474</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>1197665466</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>K-Life-Style</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>広報ジンクリーム 50ml 1個 栄養補給 ツヤ</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>多娜嫺</t>
+        </is>
+      </c>
+      <c r="F394" t="n">
+        <v>2396</v>
+      </c>
+      <c r="G394" t="n">
+        <v>1</v>
+      </c>
+      <c r="H394" t="b">
+        <v>0</v>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197665466</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>1175560636</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>seoulselectstore</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>ヘアケア マルチ ペプチド セラム フォー ヘア デンシティ 60ml</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>5720</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0</v>
+      </c>
+      <c r="H395" t="b">
+        <v>0</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175560636</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>1146350870</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>seoulselectstore</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>【NEW】 オードパルファム 08 ラブポーション 25ml</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>After blow</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>6580</v>
+      </c>
+      <c r="G396" t="n">
+        <v>0</v>
+      </c>
+      <c r="H396" t="b">
+        <v>0</v>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146350870</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>1175324790</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>transia</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>センシティブ スージング ジェルクリーム 100g ひんやりうるおい 低刺激 水分クリーム ベタつきにくい 敏感肌 朝夜兼用 オイルフリー ノンコメド印象 軽い使用感</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>2760</v>
+      </c>
+      <c r="G397" t="n">
+        <v>0</v>
+      </c>
+      <c r="H397" t="b">
+        <v>0</v>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175324790</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>1201200397</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>transia</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>アクネブレミッシュ鎮静ボディウォッシュ 460ml 背中ニキビ・肌トラブルを改善する 背中ニキビ・ボディのざらつきケア さっぱり洗浄 つっぱりにくい デイリー用</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Nodor</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>3970</v>
+      </c>
+      <c r="G398" t="n">
+        <v>3</v>
+      </c>
+      <c r="H398" t="b">
+        <v>0</v>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201200397</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J380"/>
+  <autoFilter ref="A1:J398"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 96, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$398</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$422</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J398"/>
+  <dimension ref="A1:J422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16773,8 +16773,992 @@
         </is>
       </c>
     </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>1211601601</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>JUNO_korea</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>【アヌ ア美容液】アゼライン酸10％マイルドスージングセラム 30ml(混合肌 敏感肌向け 韓国スキンケア)</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>3180</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0</v>
+      </c>
+      <c r="H399" t="b">
+        <v>0</v>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211601601</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>1209266440</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>JUNO_korea</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>【PDRN配合/リピートアイテム】ペプタシカ セラムパッド ダブルセット（60枚＋60枚）</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>トーン28</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G400" t="n">
+        <v>0</v>
+      </c>
+      <c r="H400" t="b">
+        <v>0</v>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209266440</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>1206023291</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>oreumpick</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>マジックプレス ペディキュア トマトクラッシュ 磁石ネイル 韓国 ペディチップ</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>ダッシングディバ</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G401" t="n">
+        <v>0</v>
+      </c>
+      <c r="H401" t="b">
+        <v>0</v>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206023291</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>1205988538</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>oreumpick</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>プライム プライマー セッティング フィクサー 50ml x 2個 韓国コスメ メイクキープ 韓国コスメ メイク</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F402" t="n">
+        <v>2557</v>
+      </c>
+      <c r="G402" t="n">
+        <v>2</v>
+      </c>
+      <c r="H402" t="b">
+        <v>0</v>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205988538</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>1169812368</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>coneco</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>[NEW]ラウンドアラウンド センテッド ヘア&amp;amp;ボディ ミスト 100ml</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>ROUND A ROUND</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>1618</v>
+      </c>
+      <c r="G403" t="n">
+        <v>0</v>
+      </c>
+      <c r="H403" t="b">
+        <v>0</v>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169812368</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>1155304298</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>coneco</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>ZARA 香水 HIBISCUS 90ML オードパフューム [EDP]</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>ザラ</t>
+        </is>
+      </c>
+      <c r="F404" t="n">
+        <v>4669</v>
+      </c>
+      <c r="G404" t="n">
+        <v>0</v>
+      </c>
+      <c r="H404" t="b">
+        <v>0</v>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155304298</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>1196415617</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>【WiD2】 AHA・BHA配合 28デイズヒアルクリーム (30ml) ザラつきOFF！なめらか透明肌へ 1個</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G405" t="n">
+        <v>1</v>
+      </c>
+      <c r="H405" t="b">
+        <v>0</v>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196415617</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>1196366572</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>【WiD2】 ガラクトナイアシンエッセンスマスク 10枚入り 肌をクリアに・高保湿・エイジングケア</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F406" t="n">
+        <v>2851</v>
+      </c>
+      <c r="G406" t="n">
+        <v>0</v>
+      </c>
+      <c r="H406" t="b">
+        <v>0</v>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196366572</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>1088346776</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>SnowWhiteAtelier</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>ビタペアC 生ビタミン C 美容液</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>5381</v>
+      </c>
+      <c r="G407" t="n">
+        <v>0</v>
+      </c>
+      <c r="H407" t="b">
+        <v>0</v>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1088346776</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>1120303925</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>SnowWhiteAtelier</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>【正規品】ドクダミポアディープクレンジングフォーム150ml/もちっとした泡/毛穴ディープクレンジング/角質/鎮静/8重ヒアルロン酸/保湿/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0</v>
+      </c>
+      <c r="H408" t="b">
+        <v>0</v>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1120303925</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>1098705041</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>SnowWhiteAtelier</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>【正規品/1+1/韓国皮膚科G.Uクリニック開発】PDRNリジュビネイティングクリーム 70ml/敏感肌/肌施術後鎮静/保湿/回復/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>ジェナベール</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>6526</v>
+      </c>
+      <c r="G409" t="n">
+        <v>0</v>
+      </c>
+      <c r="H409" t="b">
+        <v>0</v>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1098705041</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>1098393555</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>SnowWhiteAtelier</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>【正規品/ZB1/ Straykids Pick】クリーンウォームコットン クラシックEDP 60ml/フローラル香/シトラス香/石鹸香/韓国香水/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>クリーン</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>7104</v>
+      </c>
+      <c r="G410" t="n">
+        <v>0</v>
+      </c>
+      <c r="H410" t="b">
+        <v>0</v>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1098393555</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>1201944372</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>ライスブライトニング酵素洗顔パウダー, 40g / 韓国 人気 乾燥肌 敏感肌 米ぬか酵素洗顔クレンジング</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>3741</v>
+      </c>
+      <c r="G411" t="n">
+        <v>0</v>
+      </c>
+      <c r="H411" t="b">
+        <v>0</v>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201944372</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>1171710365</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>[NEW]PDRN 100 ヒアルロン酸 ブースター トナー 250ml, 1個 / 韓国 人気 導入化粧水 ブースター</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>3664</v>
+      </c>
+      <c r="G412" t="n">
+        <v>1</v>
+      </c>
+      <c r="H412" t="b">
+        <v>0</v>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171710365</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>1168040059</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>ドクダミ77 スージングトナー 350ml, 1個 / 韓国 人気 どくだみ 敏感肌 ニキビ 跡 赤み 鎮静 保湿 化粧水</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>4313</v>
+      </c>
+      <c r="G413" t="n">
+        <v>2</v>
+      </c>
+      <c r="H413" t="b">
+        <v>0</v>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168040059</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>1145729526</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>[大容量] ドクダミ 77 スージングトナー 350ml+詰め替え350ml / 韓国 人気 低刺激 鎮静 化粧水</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>5495</v>
+      </c>
+      <c r="G414" t="n">
+        <v>0</v>
+      </c>
+      <c r="H414" t="b">
+        <v>0</v>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145729526</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>1165988568</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>liblingz</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>【GIFT】朝鮮 美女 ジョソンビューティー 米エキス サンクリーム SPF50+/ 70ml/50ml 韓国&amp;amp;グローバル 人気/ 敏感肌向け！/ プロバイオティクス配合サンクリーム</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>1999</v>
+      </c>
+      <c r="G415" t="n">
+        <v>0</v>
+      </c>
+      <c r="H415" t="b">
+        <v>0</v>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165988568</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>1204964045</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>liblingz</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>【GIFT/リニューアル】 トリプルコラーゲントナー 4.0 / 化粧水 ハリ ツヤ インナードライハリ スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>1989</v>
+      </c>
+      <c r="G416" t="n">
+        <v>0</v>
+      </c>
+      <c r="H416" t="b">
+        <v>0</v>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204964045</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>1188839770</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>[保湿 保水 栄養 シートマスク 10枚 5種類から選択] 高保湿 まとめ買い 夜用 デイリー スキンケア</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>1709</v>
+      </c>
+      <c r="G417" t="n">
+        <v>2</v>
+      </c>
+      <c r="H417" t="b">
+        <v>0</v>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188839770</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>1197460025</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>【1+1 クリームミスト 120ml】保湿ミスト 化粧水ミスト うるおいケア 整肌ケア スプレー 韓国スキンケア デイリーケア</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G418" t="n">
+        <v>0</v>
+      </c>
+      <c r="H418" t="b">
+        <v>0</v>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197460025</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>1188077394</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>[秀麗な本超保湿クリーム 50ml] 韓国漢方 高保湿 エイジングケア シワ/改/善 /弾力アップ しっとり濃密テクスチャー</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>秀麗韓</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>4427</v>
+      </c>
+      <c r="G419" t="n">
+        <v>0</v>
+      </c>
+      <c r="H419" t="b">
+        <v>0</v>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188077394</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>1142414147</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>SKINTALKTALK</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>[NEW] ライス 4ステップ ク(レンジング パウダー +70 グロー ミルキー トナー + セラム + 70 インテンシブ モイスチャライジング ミルク)</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>10752</v>
+      </c>
+      <c r="G420" t="n">
+        <v>0</v>
+      </c>
+      <c r="H420" t="b">
+        <v>0</v>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142414147</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>1142414152</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>SKINTALKTALK</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>[NEW] ライス スキンケア 70 グロー ミルキー トナー 250ml + 250ml / うるおい×透明感！ライス70％でしっとりツヤ肌へ導くミルキートナー</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>6363</v>
+      </c>
+      <c r="G421" t="n">
+        <v>0</v>
+      </c>
+      <c r="H421" t="b">
+        <v>0</v>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142414152</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>1202885059</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>SKINTALKTALK</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>コラーゲン リフティング マスク 10枚 / ハリUP！引き締めケアでぷるツヤ肌へ</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>2885</v>
+      </c>
+      <c r="G422" t="n">
+        <v>0</v>
+      </c>
+      <c r="H422" t="b">
+        <v>0</v>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202885059</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J398"/>
+  <autoFilter ref="A1:J422"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 99, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$422</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$433</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J422"/>
+  <dimension ref="A1:J433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17757,8 +17757,459 @@
         </is>
       </c>
     </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>1183855839</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>ardistore</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>ジェイエムソリューション B5 ヒアモイスチャライジングクリーム 60ml 3本 JM 솔루션 B5 히어 모이스처라이징 크림 60ml 3병</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>4700</v>
+      </c>
+      <c r="G423" t="n">
+        <v>0</v>
+      </c>
+      <c r="H423" t="b">
+        <v>0</v>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183855839</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>1208177592</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>ardistore</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>イェジフ ヨンビン 紅参化粧品 5種 1セット 예지후 영빈 홍삼 화장품 5종 1세트</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>禮知后</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G424" t="n">
+        <v>0</v>
+      </c>
+      <c r="H424" t="b">
+        <v>0</v>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208177592</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>1172777299</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>fmalwm</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>パフューム ヘアミスト サンセットフォグ 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>ハクスリー</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>5833</v>
+      </c>
+      <c r="G425" t="n">
+        <v>0</v>
+      </c>
+      <c r="H425" t="b">
+        <v>0</v>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172777299</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>1209203301</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Mamiya</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>【シャンプー600ml * 3本+リンス600ml*3本】シャルマンマスクの香り/ケラシス パフューム/合わせて6本セット/CHARMANT MUSK/Kerasys</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G426" t="n">
+        <v>2</v>
+      </c>
+      <c r="H426" t="b">
+        <v>0</v>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209203301</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>1200038680</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Mamiya</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>【２個セット】[大容量980ml + 980ml]パフュームシャンプー+リンスセット(Lovely&amp;amp;Romantic)(Elegance&amp;amp;Sensual)香り/毛髪ツヤケア</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G427" t="n">
+        <v>0</v>
+      </c>
+      <c r="H427" t="b">
+        <v>0</v>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200038680</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>1151090202</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Mamiya</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>【シャンプー600ml * 3本+リンス600ml*3本】シャルマンマスクの香り/ケラシス パフューム/合わせて6本セット/CHARMANT MUSK/Kerasys</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G428" t="n">
+        <v>4</v>
+      </c>
+      <c r="H428" t="b">
+        <v>0</v>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151090202</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>1195242230</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>k10shop</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>イリユン セラミドアトローション 無香料 508ml 1個</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>2655</v>
+      </c>
+      <c r="G429" t="n">
+        <v>0</v>
+      </c>
+      <c r="H429" t="b">
+        <v>0</v>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195242230</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>1208323570</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>k10shop</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>SKIN1004 マダガスカルセンテラ ヒアルーシカ ウォーターフィットサンセラム 日焼け止め SPF50+ PA++++ 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>ティーゼン</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>3076</v>
+      </c>
+      <c r="G430" t="n">
+        <v>0</v>
+      </c>
+      <c r="H430" t="b">
+        <v>0</v>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208323570</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>1200677289</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>JJCompany</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>グリコール酸7% トーニングソリューション 100ml 角質ケア 拭き取り化粧水 毛穴ケア 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>2302</v>
+      </c>
+      <c r="G431" t="n">
+        <v>0</v>
+      </c>
+      <c r="H431" t="b">
+        <v>0</v>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200677289</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>1171040599</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>LUnBLOOM</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>ジェントル リフレッシング ボディウォッシュ 1L / 大容量 / 敏感肌用 / 低刺激</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>セタフィル</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G432" t="n">
+        <v>0</v>
+      </c>
+      <c r="H432" t="b">
+        <v>0</v>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171040599</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>1170913957</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>LUnBLOOM</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>キャロットカロテン モイストエフェクター55ml + キャロットカロテン リリーフクリーム 70ml / 美容液 / 水分クリーム / 潤い / 保湿 / 整肌 / 低刺激 / 鎮静 / 乾燥肌</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>5700</v>
+      </c>
+      <c r="G433" t="n">
+        <v>1</v>
+      </c>
+      <c r="H433" t="b">
+        <v>0</v>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170913957</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J422"/>
+  <autoFilter ref="A1:J433"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 102, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$433</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$441</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J433"/>
+  <dimension ref="A1:J441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18208,8 +18208,336 @@
         </is>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>1072009140</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>バイオ スキン クレンジング パッド 6g 30枚入 x 2</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>EKE</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G434" t="n">
+        <v>0</v>
+      </c>
+      <c r="H434" t="b">
+        <v>0</v>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1072009140</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>1079690675</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>CELL LINE PRO リペアクリーム [100口] 半永久化粧材料 アフターケア 1g100個入り</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Clear_pro</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G435" t="n">
+        <v>0</v>
+      </c>
+      <c r="H435" t="b">
+        <v>0</v>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1079690675</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>1062391008</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>hellojp</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>マスターズ プロパッチ 8g + 日焼け止め SPF50 + PA +++ 1.5mL 4セット</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>2164</v>
+      </c>
+      <c r="G436" t="n">
+        <v>0</v>
+      </c>
+      <c r="H436" t="b">
+        <v>0</v>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1062391008</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>1169199883</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>COCO-Beauty</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>【正規品】エッセンシャルムルマイクロフィッティングミスト, 55ml</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>ジョンセンムル</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>1808</v>
+      </c>
+      <c r="G437" t="n">
+        <v>2</v>
+      </c>
+      <c r="H437" t="b">
+        <v>0</v>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169199883</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>1170526082</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>COCO-Beauty</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>【正規品】セラミッククリーム, 100ml</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>5287</v>
+      </c>
+      <c r="G438" t="n">
+        <v>0</v>
+      </c>
+      <c r="H438" t="b">
+        <v>0</v>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170526082</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>1182429127</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>rseed</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>【PDRNマスクパック 1枚GIFT】PDRNヒアルロン酸カプセル 100セラム, 本品 30ml(シートマスク贈呈！) orレフィル 30ml 水光注射 弾力 保湿 ツヤ</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>1770</v>
+      </c>
+      <c r="G439" t="n">
+        <v>3</v>
+      </c>
+      <c r="H439" t="b">
+        <v>0</v>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182429127</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>1149457939</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>suisui</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>ポストアルファクーリングパッド70枚 / ポストアルファ シカ クーリングパッド70枚</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>2620</v>
+      </c>
+      <c r="G440" t="n">
+        <v>0</v>
+      </c>
+      <c r="H440" t="b">
+        <v>0</v>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149457939</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>1212082061</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>suisui</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>【ハローキティ限定】薬用泡ハンドソープ ギフトセット（本体 250ml + 詰め替え 200ml × 2・選べる2タイプ）</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>キレイキレイ</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>1591</v>
+      </c>
+      <c r="G441" t="n">
+        <v>1</v>
+      </c>
+      <c r="H441" t="b">
+        <v>0</v>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212082061</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J433"/>
+  <autoFilter ref="A1:J441"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 105, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$441</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$454</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J441"/>
+  <dimension ref="A1:J454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18536,8 +18536,541 @@
         </is>
       </c>
     </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>1213547055</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>トリプルシールド ハイドロロック サンセラム SPF50+ PA++++ 50ml</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Forencos</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G442" t="n">
+        <v>0</v>
+      </c>
+      <c r="H442" t="b">
+        <v>0</v>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213547055</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>1212836013</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>スキン パーフェクティング BHA リキッド エクスフォリエント 118ml + 30ml / 角質ケア 毛穴ケア ピーリング 低刺激 スキンケア</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>ポーラチョイス</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G443" t="n">
+        <v>0</v>
+      </c>
+      <c r="H443" t="b">
+        <v>0</v>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212836013</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>1211205774</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>jj_star</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>マルチペプチドトナー 50ml x 5個 / 肌保湿 / 保湿充填</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>ルネセル</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G444" t="n">
+        <v>0</v>
+      </c>
+      <c r="H444" t="b">
+        <v>0</v>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211205774</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>1210121103</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>ttonce-korea</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>ウォータープルーフ プロ サンクリーム 50g 2個 ト ラベル スポーツ日焼け止め,DEWYTREE ACディープ熱感カーミングマスク 1枚プレゼント</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>6383</v>
+      </c>
+      <c r="G445" t="n">
+        <v>0</v>
+      </c>
+      <c r="H445" t="b">
+        <v>0</v>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210121103</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>1202343508</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>ttonce-korea</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>フットパウダー 35g 3種類から1つ選択（オリジナル・オレンジ・ペパーミント）トラベル【プレゼント】シューズクリーナー3枚 足臭対策 消臭パウダー</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>GRAN'S REMEDY</t>
+        </is>
+      </c>
+      <c r="F446" t="n">
+        <v>3979</v>
+      </c>
+      <c r="G446" t="n">
+        <v>0</v>
+      </c>
+      <c r="H446" t="b">
+        <v>0</v>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202343508</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>1203741010</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>wline</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>グリーンティー ヒアルロン酸 ミスト 150ml*1本</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F447" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G447" t="n">
+        <v>0</v>
+      </c>
+      <c r="H447" t="b">
+        <v>0</v>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203741010</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>1203108224</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>wline</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>ダメージセラピーノーウォッシュトリートメント, 250mL</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>GROWUS</t>
+        </is>
+      </c>
+      <c r="F448" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G448" t="n">
+        <v>1</v>
+      </c>
+      <c r="H448" t="b">
+        <v>0</v>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203108224</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>1200335123</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>wline</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>グリーントマト ディープポア クリーン エンザイム パウダーウォッシュ 50g / 韓国化粧品</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F449" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G449" t="n">
+        <v>0</v>
+      </c>
+      <c r="H449" t="b">
+        <v>0</v>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200335123</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>1211822634</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>CinderellaBeaute</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>BOBBI BROWN(ボビイ ブラウン) ビタエンリッチド クリーム＆フェイスベース プラス 15mL</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>ボビイブラウン</t>
+        </is>
+      </c>
+      <c r="F450" t="n">
+        <v>4780</v>
+      </c>
+      <c r="G450" t="n">
+        <v>0</v>
+      </c>
+      <c r="H450" t="b">
+        <v>0</v>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211822634</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>1210078172</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>PartyTime</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>MAKE UP FOR EVER(メイクアップフォーエバー) ミスト&amp;amp;フィックス マット トラベルサイズ 30mL</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>メイクアップフォーエバー</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>2810</v>
+      </c>
+      <c r="G451" t="n">
+        <v>0</v>
+      </c>
+      <c r="H451" t="b">
+        <v>0</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210078172</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>1210785514</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>KirariSoban</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>[NEW]ボディミスト 100ml（6種択1）</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>BYREDO</t>
+        </is>
+      </c>
+      <c r="F452" t="n">
+        <v>14980</v>
+      </c>
+      <c r="G452" t="n">
+        <v>0</v>
+      </c>
+      <c r="H452" t="b">
+        <v>0</v>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210785514</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>1207285957</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>KirariSoban</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>[1+1]シグネチャー フレグランスミスト 236ml / 10種択2</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>バス&amp;amp;ボディーワークス</t>
+        </is>
+      </c>
+      <c r="F453" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G453" t="n">
+        <v>0</v>
+      </c>
+      <c r="H453" t="b">
+        <v>0</v>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207285957</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>1194955268</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>KirariSoban</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>[NEW]ヘアミスト 30ml（8種択1）</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>ディプティック</t>
+        </is>
+      </c>
+      <c r="F454" t="n">
+        <v>13578</v>
+      </c>
+      <c r="G454" t="n">
+        <v>0</v>
+      </c>
+      <c r="H454" t="b">
+        <v>0</v>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194955268</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J441"/>
+  <autoFilter ref="A1:J454"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 108, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$454</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$461</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J454"/>
+  <dimension ref="A1:J461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19069,8 +19069,295 @@
         </is>
       </c>
     </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>1208735798</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>kkbiyori</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>バハ リキッド 118ml / BHA</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>ポーラチョイス</t>
+        </is>
+      </c>
+      <c r="F455" t="n">
+        <v>4210</v>
+      </c>
+      <c r="G455" t="n">
+        <v>0</v>
+      </c>
+      <c r="H455" t="b">
+        <v>0</v>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208735798</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>1201049942</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>glowree</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>POINT ジェラートパッククレンザー 100ml</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>ダイソー</t>
+        </is>
+      </c>
+      <c r="F456" t="n">
+        <v>2190</v>
+      </c>
+      <c r="G456" t="n">
+        <v>0</v>
+      </c>
+      <c r="H456" t="b">
+        <v>0</v>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201049942</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>1196382835</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>HAPPYLADY</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>[100時間保湿/かゆみ緩和/会社員A] [正規品]シカサルブクリーム 230ml</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>MECHAI</t>
+        </is>
+      </c>
+      <c r="F457" t="n">
+        <v>5352</v>
+      </c>
+      <c r="G457" t="n">
+        <v>0</v>
+      </c>
+      <c r="H457" t="b">
+        <v>0</v>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196382835</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>1120236365</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>hangooksangin</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>ネオクラシック オムM ブラック オールインワン トリートメント 110mL メンズスキンケア 化粧水 乳液 クリーム</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>ザフェイスショップ</t>
+        </is>
+      </c>
+      <c r="F458" t="n">
+        <v>3699</v>
+      </c>
+      <c r="G458" t="n">
+        <v>0</v>
+      </c>
+      <c r="H458" t="b">
+        <v>0</v>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1120236365</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>1008962509</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Cosmo_beauty</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>[BIODERMA]センシビオジェルマウサント（クレンザー）200ml / Sensibio Gel Moussant 200ml</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>ビオデルマ</t>
+        </is>
+      </c>
+      <c r="F459" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G459" t="n">
+        <v>0</v>
+      </c>
+      <c r="H459" t="b">
+        <v>0</v>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1008962509</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>1094596934</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>hmipo</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>DASHU ダシュ プロ エアリー ポリッシュ オイル 100ml+10ml</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F460" t="n">
+        <v>3278</v>
+      </c>
+      <c r="G460" t="n">
+        <v>1</v>
+      </c>
+      <c r="H460" t="b">
+        <v>0</v>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094596934</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>1191488311</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>hmipo</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>アクアティカ サンスプレー 100mL</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F461" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G461" t="n">
+        <v>0</v>
+      </c>
+      <c r="H461" t="b">
+        <v>0</v>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191488311</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J454"/>
+  <autoFilter ref="A1:J461"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 3, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$461</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$472</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J461"/>
+  <dimension ref="A1:J472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19356,8 +19356,459 @@
         </is>
       </c>
     </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>1190126098</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>kiseki-select</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>スピケア V3エキサイティングファンデーション 15g 本体 SPICARE 韓国コスメ LOT番号付</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>SPICARE</t>
+        </is>
+      </c>
+      <c r="F462" t="n">
+        <v>4529</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0</v>
+      </c>
+      <c r="H462" t="b">
+        <v>0</v>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190126098</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>1205431137</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>kiseki-select</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>ミルボン ジェミールフラン メルティバターバーム 40g 2個セット 洗い流さない トリートメント アウトバス ハンドクリーム 美容室 サロン専売品 ミルボン milbon ヘアケア おすす</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>ミルボン</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G463" t="n">
+        <v>0</v>
+      </c>
+      <c r="H463" t="b">
+        <v>0</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205431137</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>1182162092</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>otoku-cosme</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>ナイアード ヘナ＋木藍 黒 400g Naiad 黒茶系 No.5 白髪染め ヘアカラー 染毛料 カラー剤 カラーリング 毛染め ヘナパウダー ヘナカラー ナイアードヘナ トリートメントヘアカラー 染</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>ナイアード</t>
+        </is>
+      </c>
+      <c r="F464" t="n">
+        <v>3327</v>
+      </c>
+      <c r="G464" t="n">
+        <v>1</v>
+      </c>
+      <c r="H464" t="b">
+        <v>0</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182162092</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>1200862105</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>kirei-station</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>【2個セット】チャコット フィニッシングキープミスト クール 50ml×2 メイクの仕上げや下地に使える2WAYミスト 清涼感とうるおいを与えメイクをキープ ふわふわ微細ミストの1層式 日本製</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>チャコット</t>
+        </is>
+      </c>
+      <c r="F465" t="n">
+        <v>3479</v>
+      </c>
+      <c r="G465" t="n">
+        <v>3</v>
+      </c>
+      <c r="H465" t="b">
+        <v>0</v>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200862105</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>1096984158</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>K-Blush</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>【限定特典メディヒールマスク付】プレミアム2.0 ネックスティック 20g ペプチド1000ショット 首ケア ベタつかない保湿ボリュームアップハリ 弾力 リフティング 首のしわあごのしわ韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F466" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G466" t="n">
+        <v>2</v>
+      </c>
+      <c r="H466" t="b">
+        <v>0</v>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096984158</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>1089915438</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>K-Blush</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>【公式正品】【角質ケア】グリコール酸7％ エクスフォリエーティング トナー 100ml /240mlAHA配合 拭き取り化粧水なめらか肌・キメケア・夜用スキンケア脇の黒ずみケア毛穴のざらつきケア韓国</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F467" t="n">
+        <v>2699</v>
+      </c>
+      <c r="G467" t="n">
+        <v>2</v>
+      </c>
+      <c r="H467" t="b">
+        <v>0</v>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089915438</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>1212749218</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>K-Blush</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】乳酸(Lactic Acid)10%+ヒアルロン酸HA 30ml 美容液 角質ケア 保湿 キメ なめらか肌 フェイスセラム スキンケア 韓国美容液 人気</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F468" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G468" t="n">
+        <v>0</v>
+      </c>
+      <c r="H468" t="b">
+        <v>0</v>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212749218</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>1193610404</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>LETSMILE</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸カプセル100セラム, 30ml, レフィル</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F469" t="n">
+        <v>1999</v>
+      </c>
+      <c r="G469" t="n">
+        <v>3</v>
+      </c>
+      <c r="H469" t="b">
+        <v>0</v>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193610404</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>1201075580</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>82SHOP</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>ドクダミ77 B3 ジンク トラブルセラム 美容液 30ml 1個</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F470" t="n">
+        <v>1870</v>
+      </c>
+      <c r="G470" t="n">
+        <v>0</v>
+      </c>
+      <c r="H470" t="b">
+        <v>0</v>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201075580</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>1198867352</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>82SHOP</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸 カプセルミスト 100ml 韓国コスメ 保湿ミスト 水分補給 乾燥対策</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F471" t="n">
+        <v>2520</v>
+      </c>
+      <c r="G471" t="n">
+        <v>0</v>
+      </c>
+      <c r="H471" t="b">
+        <v>0</v>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198867352</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>1158907027</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Butler_lounge</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>【ハリ＆リフティングケア】ナンバーズイン 9番 NMN BIO リフティング フルフェイスパック 4枚入り＋引き締めシート付き</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F472" t="n">
+        <v>2470</v>
+      </c>
+      <c r="G472" t="n">
+        <v>1</v>
+      </c>
+      <c r="H472" t="b">
+        <v>0</v>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158907027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J461"/>
+  <autoFilter ref="A1:J472"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 111, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$867</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$878</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J867"/>
+  <dimension ref="A1:J878"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36002,8 +36002,459 @@
         </is>
       </c>
     </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>1158685803</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>hahahaya</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>グリコリック アシッド 7% エクスポリエイティングトナー 100ml</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F868" t="n">
+        <v>1860</v>
+      </c>
+      <c r="G868" t="n">
+        <v>1</v>
+      </c>
+      <c r="H868" t="b">
+        <v>0</v>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J868" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158685803</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>1082804410</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>SuperStarK</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>【国内発送】 ターンオーバーアンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F869" t="n">
+        <v>5478</v>
+      </c>
+      <c r="G869" t="n">
+        <v>1</v>
+      </c>
+      <c r="H869" t="b">
+        <v>0</v>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J869" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1082804410</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>1198894604</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>bestone1</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>ティファニー TIFFANY ＆ラブ フォーヒム EDT + ＆ラブ フォーハー EDP ミニ香水 セット 1.2ml×2 サンプル[6495] メール便無料[B][BP3]</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Tiffany</t>
+        </is>
+      </c>
+      <c r="F870" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G870" t="n">
+        <v>1</v>
+      </c>
+      <c r="H870" t="b">
+        <v>0</v>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J870" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198894604</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>1091387881</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>バイビード インアンドアウト マスクパック,1個入り,5個,/In &amp;amp; Out Facial Mask/毛穴の老廃物を除去</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>バイビッド</t>
+        </is>
+      </c>
+      <c r="F871" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G871" t="n">
+        <v>5</v>
+      </c>
+      <c r="H871" t="b">
+        <v>0</v>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J871" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1091387881</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>1095687901</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>[KERASYS] ADVANCED KERAMIDE トリートメント！ ヘアパック！ シャンプー！ 人気商品集電線 1+1 [正規品] 韓国ブランド(鎮静/弾力/保湿/栄養供給/活力)</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F872" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G872" t="n">
+        <v>0</v>
+      </c>
+      <c r="H872" t="b">
+        <v>0</v>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J872" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1095687901</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>1101562835</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>ビフィダ バイオーム アンプル パッド 70枚</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F873" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G873" t="n">
+        <v>1</v>
+      </c>
+      <c r="H873" t="b">
+        <v>0</v>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J873" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1101562835</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>1167189098</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>GEPSTORE</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>韓国 ブラックスネイル コラーゲン ツーミスト セラム 100ml 3+3</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F874" t="n">
+        <v>11880</v>
+      </c>
+      <c r="G874" t="n">
+        <v>0</v>
+      </c>
+      <c r="H874" t="b">
+        <v>0</v>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J874" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167189098</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>1163541573</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>GEPSTORE</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>アノーブ グロウ ボディローション 290ml×2 ヌーバニラ 韓国ビューティー ボディケア</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F875" t="n">
+        <v>6780</v>
+      </c>
+      <c r="G875" t="n">
+        <v>0</v>
+      </c>
+      <c r="H875" t="b">
+        <v>0</v>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J875" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163541573</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>1106037437</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>GEPSTORE</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>ルシード エル ハイダメージ リペア ヘアオイル 90ml 髪質復元</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>ルシージェー</t>
+        </is>
+      </c>
+      <c r="F876" t="n">
+        <v>1835</v>
+      </c>
+      <c r="G876" t="n">
+        <v>0</v>
+      </c>
+      <c r="H876" t="b">
+        <v>0</v>
+      </c>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J876" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1106037437</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>1207345549</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>HELLOJ</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>1025 独島保湿ウォータージェルマスク 30ml (20個)</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F877" t="n">
+        <v>3580</v>
+      </c>
+      <c r="G877" t="n">
+        <v>0</v>
+      </c>
+      <c r="H877" t="b">
+        <v>0</v>
+      </c>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J877" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207345549</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>1205255908</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>HELLOJ</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>[1+1] クリニックテン プラス トクトクが米粒サイズの化膿性赤いスポットケア スキンクリニック10（50ml）</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>mediB</t>
+        </is>
+      </c>
+      <c r="F878" t="n">
+        <v>4850</v>
+      </c>
+      <c r="G878" t="n">
+        <v>0</v>
+      </c>
+      <c r="H878" t="b">
+        <v>0</v>
+      </c>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J878" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205255908</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J867"/>
+  <autoFilter ref="A1:J878"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 1)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$1152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$1158</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1152"/>
+  <dimension ref="A1:J1158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47687,8 +47687,254 @@
         </is>
       </c>
     </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>1174587339</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>angelrainbow</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>ブライトニング ピーリング ジェル ピーチ 100g + 100g フェイシャル スクラブ 顔 角質除去 敏感肌 低刺激 韓国 コスメ スキンケア</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>プル</t>
+        </is>
+      </c>
+      <c r="F1153" t="n">
+        <v>2659</v>
+      </c>
+      <c r="G1153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1153" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J1153" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174587339</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>1172128294</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>angelrainbow</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>コットンフット 足を洗おう フットシャンプー 385mlX2本 石鹸の香り さらさら 足 匂い ケア 韓国 スキンケア</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>オン・ザ・ボディー</t>
+        </is>
+      </c>
+      <c r="F1154" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G1154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1154" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J1154" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172128294</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>1168738382</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>angelrainbow</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>シークレット ライス 麹 ピーリング ツーフォーム クレンザー 120g デイリー 毛穴 角質 フェイシャル 洗顔 ケア キメ 低刺激 敏感肌 韓国 コスメ スキンケア</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F1155" t="n">
+        <v>4089</v>
+      </c>
+      <c r="G1155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1155" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J1155" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168738382</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>1178760167</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>toseo</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>オードパルファムスノーサイ 30ML Snow Sai</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>LIBER</t>
+        </is>
+      </c>
+      <c r="F1156" t="n">
+        <v>7430</v>
+      </c>
+      <c r="G1156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1156" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J1156" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178760167</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>1193262624</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>akiaki</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>ナンバーズイン 9番 NMN バイオ リフティング エッセンス 50ml</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>ナンバーナイン</t>
+        </is>
+      </c>
+      <c r="F1157" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G1157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1157" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J1157" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193262624</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>1212341086</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>akiaki</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>【BLACKPINK ジェニー PICK】【NEW】ヴァセリン グルタヒヤ セラム ボディローション 3種 300ml</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F1158" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G1158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1158" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J1158" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212341086</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1152"/>
+  <autoFilter ref="A1:J1158"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 1, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$266</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$289</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J266"/>
+  <dimension ref="A1:J289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11361,8 +11361,951 @@
         </is>
       </c>
     </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>1167904755</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>サロン10 ノーウォッシュトリートメント 洗い流さないトリートメント 200ml+180ml 【シナモンロールポーチ付き】</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F267" t="n">
+        <v>4050</v>
+      </c>
+      <c r="G267" t="n">
+        <v>3</v>
+      </c>
+      <c r="H267" t="b">
+        <v>0</v>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167904755</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>1207613050</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>ライティング トーンアップ サンクッションSPF50+PA+++000 / ミスティーバーブル</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>アッテ</t>
+        </is>
+      </c>
+      <c r="F268" t="n">
+        <v>3140</v>
+      </c>
+      <c r="G268" t="n">
+        <v>0</v>
+      </c>
+      <c r="H268" t="b">
+        <v>0</v>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207613050</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>1193570601</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>【コスパアンプル+ローションセット】ドクダミ80アンプル30ml + ドクダミ70 デイリーローション 200ml</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F269" t="n">
+        <v>5340</v>
+      </c>
+      <c r="G269" t="n">
+        <v>0</v>
+      </c>
+      <c r="H269" t="b">
+        <v>0</v>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193570601</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>1179238550</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>BNC</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>【レッドコスパセット】レッドブレミッシュ セラム 80ml + クリーム 70ml</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F270" t="n">
+        <v>4720</v>
+      </c>
+      <c r="G270" t="n">
+        <v>1</v>
+      </c>
+      <c r="H270" t="b">
+        <v>0</v>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179238550</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>1200477461</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Fragracy444</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>[Fragracy444] お試し香水 （原材料 アッカカッパ ホワイトモス）オーデコロン 3ml スプレーボトル 【ネコポス】</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>アッカカッパ</t>
+        </is>
+      </c>
+      <c r="F271" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G271" t="n">
+        <v>2</v>
+      </c>
+      <c r="H271" t="b">
+        <v>0</v>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200477461</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>1207667858</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Fragracy444</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>[Fragracy444] お試し香水 （原材料 タンバリンズ パフューム カモ） 1.5ml スプレーボトル 【ネコポス】</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F272" t="n">
+        <v>1180</v>
+      </c>
+      <c r="G272" t="n">
+        <v>1</v>
+      </c>
+      <c r="H272" t="b">
+        <v>0</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207667858</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>1197332981</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Fragracy444</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>[Fragracy444] お試し香水 （原材料 ルラボ テノワール 29）オードパルファム 1.5ml スプレーボトル 【ネコポス】</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LE LABO</t>
+        </is>
+      </c>
+      <c r="F273" t="n">
+        <v>1280</v>
+      </c>
+      <c r="G273" t="n">
+        <v>2</v>
+      </c>
+      <c r="H273" t="b">
+        <v>0</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197332981</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>1197332943</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Fragracy444</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>[Fragracy444] お試し香水 （原材料 キャロライナヘレラ 212 ）オーデトワレ 1.5ml スプレーボトル 【ネコポス】</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>キャロライナヘレラ</t>
+        </is>
+      </c>
+      <c r="F274" t="n">
+        <v>780</v>
+      </c>
+      <c r="G274" t="n">
+        <v>10</v>
+      </c>
+      <c r="H274" t="b">
+        <v>0</v>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197332943</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>1190403656</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>mannhattan</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>フルールドゥポー EDP 香水 1.5ml お試し 香水 dtq02A</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>ディプティック</t>
+        </is>
+      </c>
+      <c r="F275" t="n">
+        <v>999</v>
+      </c>
+      <c r="G275" t="n">
+        <v>2</v>
+      </c>
+      <c r="H275" t="b">
+        <v>0</v>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190403656</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>1150372235</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>kcstore</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>アクアスクワラン水分クリーム, 60ml+30ml, 30ml ,60ml</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>エスネイチャー</t>
+        </is>
+      </c>
+      <c r="F276" t="n">
+        <v>1555</v>
+      </c>
+      <c r="G276" t="n">
+        <v>13</v>
+      </c>
+      <c r="H276" t="b">
+        <v>0</v>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150372235</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>991027883</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>kcstore</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>RX ザ6ペプチドスキンブースターセラム 150ml</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F277" t="n">
+        <v>2134</v>
+      </c>
+      <c r="G277" t="n">
+        <v>2</v>
+      </c>
+      <c r="H277" t="b">
+        <v>0</v>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=991027883</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>1213553601</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>TOKION</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>【ピョン・ウソク アクリルスタンド付き】選べる2～3点セット シャンプー/トニック/スカルプタトゥー/メガハードスプレー/ウェットカールクリーム</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F278" t="n">
+        <v>4187</v>
+      </c>
+      <c r="G278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="b">
+        <v>0</v>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213553601</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>1213380154</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>TOKION</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Stray Kids ストレイキッズ SKZ 公式ペンライト OFFICIAL LIGHT STICK ver.2</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>JYP Entertainment</t>
+        </is>
+      </c>
+      <c r="F279" t="n">
+        <v>6890</v>
+      </c>
+      <c r="G279" t="n">
+        <v>0</v>
+      </c>
+      <c r="H279" t="b">
+        <v>0</v>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213380154</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>1107382665</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>glowm</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>ダーマ HPC 水分カーミングマスクパック　10枚</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Glow.M</t>
+        </is>
+      </c>
+      <c r="F280" t="n">
+        <v>8500</v>
+      </c>
+      <c r="G280" t="n">
+        <v>5</v>
+      </c>
+      <c r="H280" t="b">
+        <v>0</v>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1107382665</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>1194978904</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>bireistore</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>【正規品＆国内発送】【lalachuu/ララチュー】ヘアファンデーション プレミアムEX ダークブラウン レフィル(パフ付き) 日本限定 発色密着持続性アップ 71種類の美容成分配合 1品5役 薄毛</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>lala chuu</t>
+        </is>
+      </c>
+      <c r="F281" t="n">
+        <v>4350</v>
+      </c>
+      <c r="G281" t="n">
+        <v>3</v>
+      </c>
+      <c r="H281" t="b">
+        <v>0</v>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194978904</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>1194975406</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>bireistore</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>【正規品＆国内発送】【lalachuu/ララチュー】ヘアファンデーション プレミアムEX ダークブラウン 本品 コンパクト付き 日本限定 発色密着持続性アップ 71種類の美容成分配合 1品5役 薄毛</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>lala chuu</t>
+        </is>
+      </c>
+      <c r="F282" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G282" t="n">
+        <v>0</v>
+      </c>
+      <c r="H282" t="b">
+        <v>0</v>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194975406</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>1202277840</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>medianswer</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>【公式】ビタコラーゲン ナノショット ハイドロゲルマスク, 5枚 3種コラーゲン 10種ビタミン 超低分子100Da 浸透ケア ツヤ 透明感 ハリ 毛穴ケア 保湿 密着 フェイスパック 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F283" t="n">
+        <v>3260</v>
+      </c>
+      <c r="G283" t="n">
+        <v>0</v>
+      </c>
+      <c r="H283" t="b">
+        <v>0</v>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202277840</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>1203559783</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>medianswer</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>【公式】【選べるナノショットハイドロゲルマスク特集】ビタコラーゲン・ポアコラーゲン・カーミングコラーゲン・リアルスキンフィットコラーゲン 10枚入り 密着保湿 フェイスパック 韓国</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F284" t="n">
+        <v>6520</v>
+      </c>
+      <c r="G284" t="n">
+        <v>2</v>
+      </c>
+      <c r="H284" t="b">
+        <v>0</v>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203559783</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>1202308494</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>medianswer</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>【公式】ポアコラーゲン ナノショット ハイドロゲルマスク 5枚 /超低分子100Da / ポアコンプレックス /毛穴ケア / キメ / ハリ/ 保湿 / 密着 / フェイスパック / 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F285" t="n">
+        <v>3260</v>
+      </c>
+      <c r="G285" t="n">
+        <v>0</v>
+      </c>
+      <c r="H285" t="b">
+        <v>0</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202308494</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>1202098452</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>medianswer</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>【公式】 レチノイドリフトシルマスク, 4枚 /チノールマスク / ハリケア / 密着 / 保湿 / ハイドロゲル / フェイスパック / 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F286" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G286" t="n">
+        <v>0</v>
+      </c>
+      <c r="H286" t="b">
+        <v>0</v>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202098452</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>1135307770</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>medianswer_japan</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>コラーゲンマスク　ポア　10枚入り 使用期限(~2026/10/15) 　毛穴　引き締め　収斂　寝たままパック　寝たままマスク　消えるマスク</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>MediAnswer</t>
+        </is>
+      </c>
+      <c r="F287" t="n">
+        <v>3630</v>
+      </c>
+      <c r="G287" t="n">
+        <v>5</v>
+      </c>
+      <c r="H287" t="b">
+        <v>0</v>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135307770</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>1026432127</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>cread_inc</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>グランズレメディ 50ｇ 正規品 単品 靴 消臭 粉 魔法の粉 足 匂い 臭い スニーカー ブーツ 下駄箱 モアビビ パウダー 無香料 クールミント フローラル</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>GRAN'S REMEDY</t>
+        </is>
+      </c>
+      <c r="F288" t="n">
+        <v>3248</v>
+      </c>
+      <c r="G288" t="n">
+        <v>16</v>
+      </c>
+      <c r="H288" t="b">
+        <v>0</v>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1026432127</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>1197142140</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>cread_inc</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>プロ業務用 UVスプレー氷冷 日焼け止め 冷感 冷却 スプレー 日焼け止め クール 紫外線対策 敏感肌 UVスプレー 全身 顔 髪 頭皮 体 保湿</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>ヤーマン</t>
+        </is>
+      </c>
+      <c r="F289" t="n">
+        <v>1760</v>
+      </c>
+      <c r="G289" t="n">
+        <v>0</v>
+      </c>
+      <c r="H289" t="b">
+        <v>0</v>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197142140</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J266"/>
+  <autoFilter ref="A1:J289"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 2, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$311</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J294"/>
+  <dimension ref="A1:J311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12509,8 +12509,705 @@
         </is>
       </c>
     </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>1191320300</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>frommedi</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>アズレンシカカーミングマスク（16枚） / トラブル鎮静 / ナイトパック</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>フロムメディ</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>11400</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0</v>
+      </c>
+      <c r="H295" t="b">
+        <v>0</v>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191320300</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>1108626331</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>helenpark_korea</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>[公式代理店]3個setで集中シワケア! ジェラシアンクリーム75ml 主成分アデノシンがほうれい線シワに効く！</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>ヘレンパーク</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>6900</v>
+      </c>
+      <c r="G296" t="n">
+        <v>4</v>
+      </c>
+      <c r="H296" t="b">
+        <v>0</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1108626331</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>1108620460</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>helenpark_korea</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>[公式代理店] 3個セット ピュアソブリン200ml お肌の悩みを一気に解消! これひとつで基礎化粧完了! 話題の韓国コスメ!</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>ヘレンパーク</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>6890</v>
+      </c>
+      <c r="G297" t="n">
+        <v>1</v>
+      </c>
+      <c r="H297" t="b">
+        <v>0</v>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1108620460</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>1108619590</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>helenpark_korea</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>[公式代理店] ピュアソブリン200ml お肌の悩みを一気に解消! これひとつで基礎化粧完了! 話題の韓国コスメ!</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>ヘレンパーク</t>
+        </is>
+      </c>
+      <c r="F298" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G298" t="n">
+        <v>1</v>
+      </c>
+      <c r="H298" t="b">
+        <v>0</v>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1108619590</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>1210642143</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>【2個セット】ミルボン エマルジョン+ 120g アウトバストリートメント ヘアミルク 洗い流さないトリートメント 太い髪 硬い髪 保湿 ヘアケア</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>エルジューダ</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>4289</v>
+      </c>
+      <c r="G299" t="n">
+        <v>0</v>
+      </c>
+      <c r="H299" t="b">
+        <v>0</v>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210642143</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>1210641925</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>ryugaichinomiya</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>【2個セット】ミルボン エマルジョン 120g アウトバストリートメント ヘアミルク 洗い流さないトリートメント 太い髪 硬い髪 保湿 ヘアケア</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>エルジューダ</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>4289</v>
+      </c>
+      <c r="G300" t="n">
+        <v>1</v>
+      </c>
+      <c r="H300" t="b">
+        <v>0</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210641925</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>1210642039</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>lwcompany</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>【2個セット】ミルボン エマルジョン+ 120g アウトバストリートメント ヘアミルク 洗い流さないトリートメント 太い髪 硬い髪 保湿 ヘアケア</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>エルジューダ</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>4289</v>
+      </c>
+      <c r="G301" t="n">
+        <v>1</v>
+      </c>
+      <c r="H301" t="b">
+        <v>0</v>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210642039</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>1180727538</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>lifemato2</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>【1+1】 ADBeLLus glowup PDRN シートマスク パック サーモン ナイアシンアミド レチノール アゼライン酸 オールインワン ギフト プレゼント フェイスマスク 大容量 30枚</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>ADBeLLus</t>
+        </is>
+      </c>
+      <c r="F302" t="n">
+        <v>1780</v>
+      </c>
+      <c r="G302" t="n">
+        <v>6</v>
+      </c>
+      <c r="H302" t="b">
+        <v>0</v>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180727538</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>1119220280</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>lifemato2</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>MDSKIN LABO シートマスク パック グルタチオン アルブチン セラミド フェイスマスク フェイスパック オールインワン 保湿 30枚入り</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>MDSKIN LABO</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>899</v>
+      </c>
+      <c r="G303" t="n">
+        <v>4</v>
+      </c>
+      <c r="H303" t="b">
+        <v>0</v>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1119220280</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>1086136823</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>lifemato2</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>【1+1】 MDSKIN LABO シートマスク パック フェイスマスク フェイスパック CICA シカ ツボクサ オールインワン ヒアルロン酸 プラセンタ スクワラン 30枚</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>MDSKIN LABO</t>
+        </is>
+      </c>
+      <c r="F304" t="n">
+        <v>1580</v>
+      </c>
+      <c r="G304" t="n">
+        <v>12</v>
+      </c>
+      <c r="H304" t="b">
+        <v>0</v>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1086136823</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>1152642613</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>shikishima</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>エルジューダ エマルジョン 120g 細髪用 ヘアケア 洗い流さない トリートメント</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>ミルボン</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G305" t="n">
+        <v>14</v>
+      </c>
+      <c r="H305" t="b">
+        <v>0</v>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152642613</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>1049534463</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>importjack</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>サンオイル ダーク タンニングオイル 180ml SPF4　日焼けオイル 日焼けローション 小麦肌 最強 日焼け メンズ 人気 タンニング サンケア BLACKKONG</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>BLACKKONG</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G306" t="n">
+        <v>4</v>
+      </c>
+      <c r="H306" t="b">
+        <v>0</v>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1049534463</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>1192121092</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>importjack</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>【国内正規品】 TL-B タイトニング アイセラム 30ml エイジングケア 目もと専用 目元ケア アイクリームしわ 取り しわ取り しわ改善 ハリ 潤い 目元クリーム</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>ストリベクチン</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>5940</v>
+      </c>
+      <c r="G307" t="n">
+        <v>1</v>
+      </c>
+      <c r="H307" t="b">
+        <v>0</v>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192121092</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>1188353289</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>importjack</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>【国内正規品】 ハードウエァ シャイン トップコート 6ml butter LONDON プロ仕上げ プロ仕上げ 高光沢トップコートハードトップコート</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>バターロンドン</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>2002</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" t="b">
+        <v>0</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188353289</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>1099357679</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>importjack</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>【スプレーノズル付】 サンオイル ゴールデン＆ダーク 2本セット 日焼けオイル 日焼けローション 真っ黒 日焼け タンニング BLACKKONG</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>BLACKKONG</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="b">
+        <v>0</v>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1099357679</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>1105768411</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>importjack</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>医師監修 ラクトバチルス乳酸菌 配合　オンプ　フェミニン潤いジェル 12本入り 　女性用　潤滑ジェル 潤滑ゼリー　フェムケア　デリケートゾーンケア　膣ケア インナージェル 日本製</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>on'peut</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>3520</v>
+      </c>
+      <c r="G310" t="n">
+        <v>19</v>
+      </c>
+      <c r="H310" t="b">
+        <v>0</v>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1105768411</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>1124209819</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>puril</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>[女性の親密な香水] 韓国コスメ インナー パフューム デリケートゾーン フェミニンウォッシュ インナー香水 生理臭い除去 インナーパフューム5ml</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Puri L</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G311" t="n">
+        <v>5</v>
+      </c>
+      <c r="H311" t="b">
+        <v>0</v>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1124209819</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J294"/>
+  <autoFilter ref="A1:J311"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 7, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$345</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$346</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J345"/>
+  <dimension ref="A1:J346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14600,8 +14600,49 @@
         </is>
       </c>
     </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>1109206240</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>hayejin</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>【送料無料】99.9％ライスフィラフェイスオイル 30ml / ライスブランオイル /美容オイル / 化粧水 / 美容液 / 米ぬか油 / マッサージオイル / ヴィーガンコスメ</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>ハイェジン</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G346" t="n">
+        <v>19</v>
+      </c>
+      <c r="H346" t="b">
+        <v>0</v>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109206240</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J345"/>
+  <autoFilter ref="A1:J346"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 8, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$346</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$348</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J346"/>
+  <dimension ref="A1:J348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14641,8 +14641,90 @@
         </is>
       </c>
     </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>1180316824</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>kjodal</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>トリートメントエンザイムクレンジングフォーム(31g*3ea)</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>アモーレパシフィック</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>1790</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0</v>
+      </c>
+      <c r="H347" t="b">
+        <v>0</v>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180316824</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>1180316719</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>kjodal</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>トリートメントエンザイムクレンジングフォーム 120g</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>アモーレパシフィック</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0</v>
+      </c>
+      <c r="H348" t="b">
+        <v>0</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180316719</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J346"/>
+  <autoFilter ref="A1:J348"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 5)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$358</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$359</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J358"/>
+  <dimension ref="A1:J359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15133,8 +15133,49 @@
         </is>
       </c>
     </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>1207194443</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>summerseve</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>公式 フェミニンウォッシュ ホワイトリリー 237ml 着色料フリー パラベンフリー デリケートゾーン におい ニオイ ムレ 蒸れ summers eve logi</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>サマーズイブ</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>1188</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0</v>
+      </c>
+      <c r="H359" t="b">
+        <v>0</v>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207194443</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J358"/>
+  <autoFilter ref="A1:J359"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 6)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$359</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$361</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J359"/>
+  <dimension ref="A1:J361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15174,8 +15174,90 @@
         </is>
       </c>
     </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>1207298644</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>fomienne</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>【公式】デリケートゾーン ミスト 30ml フェムケア ニオイケア pHバランス 弱酸性 インナーパフューム フォミエンヌ</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Fomienne</t>
+        </is>
+      </c>
+      <c r="F360" t="n">
+        <v>2370</v>
+      </c>
+      <c r="G360" t="n">
+        <v>1</v>
+      </c>
+      <c r="H360" t="b">
+        <v>0</v>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207298644</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>1197145904</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>fomienne</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>【公式】デリケートゾーン 保湿ジェル 500ml 大容量 低刺激 敏感肌 ボディジェル フェムケア フォミエンヌ</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Fomienne</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0</v>
+      </c>
+      <c r="H361" t="b">
+        <v>0</v>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197145904</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J359"/>
+  <autoFilter ref="A1:J361"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 7)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$369</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J361"/>
+  <dimension ref="A1:J369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15256,8 +15256,336 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>981403967</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>ocjapan</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>スキンバランシングトナー 300ml</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>オキシジェンシューティカルズ</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>5280</v>
+      </c>
+      <c r="G362" t="n">
+        <v>9</v>
+      </c>
+      <c r="H362" t="b">
+        <v>0</v>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=981403967</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>1094821994</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>ocjapan</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>ニュートリエントトナー 1000ml</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>オキシジェンシューティカルズ</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>14300</v>
+      </c>
+      <c r="G363" t="n">
+        <v>12</v>
+      </c>
+      <c r="H363" t="b">
+        <v>0</v>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094821994</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>1034770647</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>ocjapan</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>HAジェル (50ml)</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>オキシジェンシューティカルズ</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>7260</v>
+      </c>
+      <c r="G364" t="n">
+        <v>5</v>
+      </c>
+      <c r="H364" t="b">
+        <v>0</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1034770647</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>984241939</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>ocjapan</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>潤いツヤ肌美容液セット(50ml/50ml)</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>オキシジェンシューティカルズ</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>18700</v>
+      </c>
+      <c r="G365" t="n">
+        <v>14</v>
+      </c>
+      <c r="H365" t="b">
+        <v>0</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=984241939</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>984239343</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>ocjapan</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>弾力ケア水光美容液セット(50ml/50ml)</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>オキシジェンシューティカルズ</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>18700</v>
+      </c>
+      <c r="G366" t="n">
+        <v>12</v>
+      </c>
+      <c r="H366" t="b">
+        <v>0</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=984239343</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>1106587131</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>drmedion</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>スパオキシデュアルジェルVCプラス 100g【スプレー式炭酸パック】</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Dr. MEDION</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G367" t="n">
+        <v>7</v>
+      </c>
+      <c r="H367" t="b">
+        <v>0</v>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1106587131</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>1097625068</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>drmedion</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>スパオキシフォーミングウォッシュ【濃密炭酸泡洗顔】150g 3本セット</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Dr. MEDION</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>9460</v>
+      </c>
+      <c r="G368" t="n">
+        <v>13</v>
+      </c>
+      <c r="H368" t="b">
+        <v>0</v>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097625068</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>1066645310</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>drmedion</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>スパオキシフォーミングウォッシュ【濃密炭酸泡洗顔】150g（約1-1.5ヶ月分）</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Dr. MEDION</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>3520</v>
+      </c>
+      <c r="G369" t="n">
+        <v>16</v>
+      </c>
+      <c r="H369" t="b">
+        <v>0</v>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1066645310</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J361"/>
+  <autoFilter ref="A1:J369"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 4, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$378</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$379</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J378"/>
+  <dimension ref="A1:J379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15953,8 +15953,49 @@
         </is>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>1187917467</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Lassieel</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>明日葉 鎮静エイジング シートマスク</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Lassie'el</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>445</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0</v>
+      </c>
+      <c r="H379" t="b">
+        <v>0</v>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187917467</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J378"/>
+  <autoFilter ref="A1:J379"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 9 own-file progress (반복 5, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_9.xlsx
+++ b/output/discovery_result_9.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$389</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$392</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J389"/>
+  <dimension ref="A1:J392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16404,8 +16404,131 @@
         </is>
       </c>
     </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>1208816410</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>BULK_HOMME</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>【公式】洗顔料 メンズ THE FACE WASH 100g 泡洗顔 クレンジング 毛穴 皮脂 黒ずみ 角質 乾燥 敏感肌 メンズスキンケア ギフト</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>バルクオム</t>
+        </is>
+      </c>
+      <c r="F390" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0</v>
+      </c>
+      <c r="H390" t="b">
+        <v>0</v>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208816410</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>1208817740</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>BULK_HOMME</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>【公式】ヘアオイル メンズ 70mL 洗い流さないトリートメント くせ毛 まとまり ツヤ フローラルフルーティの香り メンズヘアケア ギフト</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>バルクオム</t>
+        </is>
+      </c>
+      <c r="F391" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G391" t="n">
+        <v>0</v>
+      </c>
+      <c r="H391" t="b">
+        <v>0</v>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208817740</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>1208862280</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>BULK_HOMME</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>【公式】洗顔料 100g &amp;amp; 泡立てネット セット メンズ 泡洗顔 クレンジング 毛穴 皮脂 黒ずみ 角質 メンズスキンケア ギフト</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>バルクオム</t>
+        </is>
+      </c>
+      <c r="F392" t="n">
+        <v>3146</v>
+      </c>
+      <c r="G392" t="n">
+        <v>0</v>
+      </c>
+      <c r="H392" t="b">
+        <v>0</v>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208862280</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J389"/>
+  <autoFilter ref="A1:J392"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>